<commit_message>
Anchor FY2027 base case to Nike's October 2026 guidance
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165EZvQ75cJkxj7zQj4acn5
</commit_message>
<xml_diff>
--- a/nike_forecast_model.xlsx
+++ b/nike_forecast_model.xlsx
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">The forecast assumptions are my own judgement for this exercise, not company guidance.</t>
+    <t xml:space="preserve">The FY2027 base case is set to match Nike's guidance of 1 Oct 2026 (revenue down a high single digit percentage, EPS of about $1.15 to $1.35 before restructuring). The regional split and FY2028 to FY2031 are my own assumptions.</t>
   </si>
   <si>
     <t xml:space="preserve">Colour key</t>
@@ -1269,19 +1269,19 @@
                   <c:v>46398</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>47184.99</c:v>
+                  <c:v>42441.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>48859.2816</c:v>
+                  <c:v>43237.0646</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>51025.774188</c:v>
+                  <c:v>45140.246492</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>53113.39418592</c:v>
+                  <c:v>47196.84009108</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>55144.7183984496</c:v>
+                  <c:v>49129.9747031382</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1289,11 +1289,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="93230587"/>
-        <c:axId val="19965658"/>
+        <c:axId val="34197154"/>
+        <c:axId val="46755491"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93230587"/>
+        <c:axId val="34197154"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1325,7 +1325,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19965658"/>
+        <c:crossAx val="46755491"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1333,7 +1333,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19965658"/>
+        <c:axId val="46755491"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1376,7 +1376,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93230587"/>
+        <c:crossAx val="34197154"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1549,19 +1549,19 @@
                   <c:v>0.0818354239406871</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0869999999999999</c:v>
+                  <c:v>0.047</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.0970000000000001</c:v>
+                  <c:v>0.0679999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.107</c:v>
+                  <c:v>0.0860000000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.115</c:v>
+                  <c:v>0.0999999999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.117</c:v>
+                  <c:v>0.111</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1576,11 +1576,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47797936"/>
-        <c:axId val="40498576"/>
+        <c:axId val="52383983"/>
+        <c:axId val="36317351"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47797936"/>
+        <c:axId val="52383983"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1612,7 +1612,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40498576"/>
+        <c:crossAx val="36317351"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1620,7 +1620,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40498576"/>
+        <c:axId val="36317351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1663,7 +1663,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47797936"/>
+        <c:crossAx val="52383983"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1836,19 +1836,19 @@
                   <c:v>46398</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>48322.56</c:v>
+                  <c:v>43972.33</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>51202.4394</c:v>
+                  <c:v>45896.7335</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>54550.232238</c:v>
+                  <c:v>48888.269</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>57724.64098332</c:v>
+                  <c:v>51733.11104025</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>60509.7100147308</c:v>
+                  <c:v>54367.378408842</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1956,19 +1956,19 @@
                   <c:v>46398</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>47184.99</c:v>
+                  <c:v>42441.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48859.2816</c:v>
+                  <c:v>43237.0646</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>51025.774188</c:v>
+                  <c:v>45140.246492</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>53113.39418592</c:v>
+                  <c:v>47196.84009108</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>55144.7183984496</c:v>
+                  <c:v>49129.9747031382</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2076,19 +2076,19 @@
                   <c:v>46398</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45376.28</c:v>
+                  <c:v>40852.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45466.6719</c:v>
+                  <c:v>40101.8204</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46014.030922</c:v>
+                  <c:v>40556.214724</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46884.9837473</c:v>
+                  <c:v>41522.70563568</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>47822.6648523902</c:v>
+                  <c:v>42553.7490738336</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2103,11 +2103,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="13353236"/>
-        <c:axId val="72335449"/>
+        <c:axId val="74369079"/>
+        <c:axId val="72168215"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="13353236"/>
+        <c:axId val="74369079"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2139,7 +2139,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72335449"/>
+        <c:crossAx val="72168215"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2147,7 +2147,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72335449"/>
+        <c:axId val="72168215"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="35000"/>
@@ -2190,7 +2190,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13353236"/>
+        <c:crossAx val="74369079"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2761,23 +2761,23 @@
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">'Income Statement'!E5</f>
-        <v>47184.99</v>
+        <v>42441.5</v>
       </c>
       <c r="F5" s="10" t="n">
         <f aca="false">'Income Statement'!F5</f>
-        <v>48859.2816</v>
+        <v>43237.0646</v>
       </c>
       <c r="G5" s="10" t="n">
         <f aca="false">'Income Statement'!G5</f>
-        <v>51025.774188</v>
+        <v>45140.246492</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">'Income Statement'!H5</f>
-        <v>53113.39418592</v>
+        <v>47196.84009108</v>
       </c>
       <c r="I5" s="10" t="n">
         <f aca="false">'Income Statement'!I5</f>
-        <v>55144.7183984496</v>
+        <v>49129.9747031382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2795,23 +2795,23 @@
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">'Revenue Build'!E20</f>
-        <v>0.0169617224880383</v>
+        <v>-0.0852730721151774</v>
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">'Revenue Build'!F20</f>
-        <v>0.0354835637349928</v>
+        <v>0.0187449689572707</v>
       </c>
       <c r="G6" s="12" t="n">
         <f aca="false">'Revenue Build'!G20</f>
-        <v>0.0443414744763664</v>
+        <v>0.0440173705039171</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">'Revenue Build'!H20</f>
-        <v>0.0409130489667506</v>
+        <v>0.0455600879238549</v>
       </c>
       <c r="I6" s="12" t="n">
         <f aca="false">'Revenue Build'!I20</f>
-        <v>0.0382450461632913</v>
+        <v>0.0409589838711164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2832,19 +2832,19 @@
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">'Income Statement'!E22</f>
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">'Income Statement'!F22</f>
-        <v>0.435</v>
+        <v>0.43</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">'Income Statement'!G22</f>
-        <v>0.44</v>
+        <v>0.435</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">'Income Statement'!H22</f>
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="I7" s="12" t="n">
         <f aca="false">'Income Statement'!I22</f>
@@ -2869,23 +2869,23 @@
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">'Income Statement'!E10</f>
-        <v>4105.09413</v>
+        <v>1994.7505</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">'Income Statement'!F10</f>
-        <v>4739.35031520001</v>
+        <v>2940.1203928</v>
       </c>
       <c r="G8" s="10" t="n">
         <f aca="false">'Income Statement'!G10</f>
-        <v>5459.757838116</v>
+        <v>3882.061198312</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">'Income Statement'!H10</f>
-        <v>6108.04033138081</v>
+        <v>4719.684009108</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">'Income Statement'!I10</f>
-        <v>6451.93205261861</v>
+        <v>5453.42719204834</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2906,23 +2906,23 @@
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">'Income Statement'!E25</f>
-        <v>0.0869999999999999</v>
+        <v>0.047</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">'Income Statement'!F25</f>
-        <v>0.0970000000000001</v>
+        <v>0.0679999999999999</v>
       </c>
       <c r="G9" s="12" t="n">
         <f aca="false">'Income Statement'!G25</f>
-        <v>0.107</v>
+        <v>0.0860000000000001</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">'Income Statement'!H25</f>
-        <v>0.115</v>
+        <v>0.0999999999999999</v>
       </c>
       <c r="I9" s="12" t="n">
         <f aca="false">'Income Statement'!I25</f>
-        <v>0.117</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2943,23 +2943,23 @@
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">'Income Statement'!E15</f>
-        <v>3323.7208953</v>
+        <v>1614.342555</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">'Income Statement'!F15</f>
-        <v>3874.92795691624</v>
+        <v>2405.86606513503</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">'Income Statement'!G15</f>
-        <v>4465.8093254168</v>
+        <v>3175.05498876406</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">'Income Statement'!H15</f>
-        <v>4998.89045250008</v>
+        <v>3857.44867124394</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">'Income Statement'!I15</f>
-        <v>5275.91483393109</v>
+        <v>4437.15300970018</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,23 +2980,23 @@
       </c>
       <c r="E11" s="14" t="n">
         <f aca="false">'Income Statement'!E18</f>
-        <v>2.25235208626609</v>
+        <v>1.08874898330804</v>
       </c>
       <c r="F11" s="14" t="n">
         <f aca="false">'Income Statement'!F18</f>
-        <v>2.65952502190545</v>
+        <v>1.63210994299397</v>
       </c>
       <c r="G11" s="14" t="n">
         <f aca="false">'Income Statement'!G18</f>
-        <v>3.11930802706645</v>
+        <v>2.18655149871843</v>
       </c>
       <c r="H11" s="14" t="n">
         <f aca="false">'Income Statement'!H18</f>
-        <v>3.57148639140278</v>
+        <v>2.72682749304722</v>
       </c>
       <c r="I11" s="14" t="n">
         <f aca="false">'Income Statement'!I18</f>
-        <v>3.87649877584944</v>
+        <v>3.23259503871925</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3017,23 +3017,23 @@
       </c>
       <c r="E12" s="10" t="n">
         <f aca="false">'Cash Flow'!E15</f>
-        <v>5308.81870790274</v>
+        <v>3962.32607554795</v>
       </c>
       <c r="F12" s="10" t="n">
         <f aca="false">'Cash Flow'!F15</f>
-        <v>5651.76603637377</v>
+        <v>4056.84168707476</v>
       </c>
       <c r="G12" s="10" t="n">
         <f aca="false">'Cash Flow'!G15</f>
-        <v>6291.20850642786</v>
+        <v>4791.29072001118</v>
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">'Cash Flow'!H15</f>
-        <v>6560.96877858743</v>
+        <v>5225.69238113624</v>
       </c>
       <c r="I12" s="10" t="n">
         <f aca="false">'Cash Flow'!I15</f>
-        <v>6796.4601261587</v>
+        <v>5809.4681678019</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3054,23 +3054,23 @@
       </c>
       <c r="E13" s="10" t="n">
         <f aca="false">'Cash Flow'!E35</f>
-        <v>4553.85886790274</v>
+        <v>3283.26207554795</v>
       </c>
       <c r="F13" s="10" t="n">
         <f aca="false">'Cash Flow'!F35</f>
-        <v>4870.01753077377</v>
+        <v>3365.04865347476</v>
       </c>
       <c r="G13" s="10" t="n">
         <f aca="false">'Cash Flow'!G35</f>
-        <v>5474.79611941986</v>
+        <v>4069.04677613918</v>
       </c>
       <c r="H13" s="10" t="n">
         <f aca="false">'Cash Flow'!H35</f>
-        <v>5711.15447161271</v>
+        <v>4470.54293967896</v>
       </c>
       <c r="I13" s="10" t="n">
         <f aca="false">'Cash Flow'!I35</f>
-        <v>5914.14463178351</v>
+        <v>5023.38857255169</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3091,23 +3091,23 @@
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">'Cash Flow'!E36</f>
-        <v>3518.24858203916</v>
+        <v>2659.84419311276</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">'Cash Flow'!F36</f>
-        <v>4610.71330013504</v>
+        <v>3145.75866531623</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">'Cash Flow'!G36</f>
-        <v>5193.58597695814</v>
+        <v>3930.80318759847</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">'Cash Flow'!H36</f>
-        <v>5765.04910200456</v>
+        <v>4986.50906756031</v>
       </c>
       <c r="I14" s="10" t="n">
         <f aca="false">'Cash Flow'!I36</f>
-        <v>6323.09603659415</v>
+        <v>5533.31945068174</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3128,23 +3128,23 @@
       </c>
       <c r="E15" s="10" t="n">
         <f aca="false">'Balance Sheet'!E6+'Balance Sheet'!E7</f>
-        <v>8062.61028586357</v>
+        <v>7650.41788243518</v>
       </c>
       <c r="F15" s="10" t="n">
         <f aca="false">'Balance Sheet'!F6+'Balance Sheet'!F7</f>
-        <v>8321.9145165023</v>
+        <v>7869.70787059372</v>
       </c>
       <c r="G15" s="10" t="n">
         <f aca="false">'Balance Sheet'!G6+'Balance Sheet'!G7</f>
-        <v>8603.12465896403</v>
+        <v>8007.95145913443</v>
       </c>
       <c r="H15" s="10" t="n">
         <f aca="false">'Balance Sheet'!H6+'Balance Sheet'!H7</f>
-        <v>8549.23002857218</v>
+        <v>7491.98533125308</v>
       </c>
       <c r="I15" s="10" t="n">
         <f aca="false">'Balance Sheet'!I6+'Balance Sheet'!I7</f>
-        <v>8140.27862376154</v>
+        <v>6982.05445312302</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3300,11 +3300,11 @@
       <c r="D9" s="19"/>
       <c r="E9" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E16,E23,E30)</f>
-        <v>0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="F9" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F16,F23,F30)</f>
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G9" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G16,G23,G30)</f>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="H9" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,H16,H23,H30)</f>
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="I9" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,I16,I23,I30)</f>
@@ -3328,11 +3328,11 @@
       <c r="D10" s="19"/>
       <c r="E10" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E17,E24,E31)</f>
-        <v>0.02</v>
+        <v>-0.08</v>
       </c>
       <c r="F10" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F17,F24,F31)</f>
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="G10" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G17,G24,G31)</f>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="I10" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,I17,I24,I31)</f>
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3356,11 +3356,11 @@
       <c r="D11" s="19"/>
       <c r="E11" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E18,E25,E32)</f>
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F18,F25,F32)</f>
-        <v>0</v>
+        <v>-0.03</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G18,G25,G32)</f>
@@ -3384,11 +3384,11 @@
       <c r="D12" s="19"/>
       <c r="E12" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E19,E26,E33)</f>
-        <v>0.02</v>
+        <v>-0.06</v>
       </c>
       <c r="F12" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F19,F26,F33)</f>
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="G12" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G19,G26,G33)</f>
@@ -3412,15 +3412,15 @@
       <c r="D13" s="19"/>
       <c r="E13" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E20,E27,E34)</f>
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="F13" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F20,F27,F34)</f>
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="G13" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G20,G27,G34)</f>
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H13" s="20" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,H20,H27,H34)</f>
@@ -3452,16 +3452,16 @@
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
       <c r="E16" s="21" t="n">
-        <v>0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G16" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="I16" s="21" t="n">
         <v>0.04</v>
@@ -3475,10 +3475,10 @@
       <c r="C17" s="19"/>
       <c r="D17" s="19"/>
       <c r="E17" s="21" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="F17" s="21" t="n">
         <v>0.02</v>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.03</v>
       </c>
       <c r="G17" s="21" t="n">
         <v>0.04</v>
@@ -3487,7 +3487,7 @@
         <v>0.04</v>
       </c>
       <c r="I17" s="21" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3498,10 +3498,10 @@
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
       <c r="E18" s="21" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>0</v>
+        <v>-0.03</v>
       </c>
       <c r="G18" s="21" t="n">
         <v>0.03</v>
@@ -3521,10 +3521,10 @@
       <c r="C19" s="19"/>
       <c r="D19" s="19"/>
       <c r="E19" s="21" t="n">
-        <v>0.02</v>
+        <v>-0.06</v>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="G19" s="21" t="n">
         <v>0.05</v>
@@ -3544,13 +3544,13 @@
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
       <c r="E20" s="21" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="F20" s="21" t="n">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="G20" s="21" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H20" s="21" t="n">
         <v>0.02</v>
@@ -3580,10 +3580,10 @@
       <c r="C23" s="19"/>
       <c r="D23" s="19"/>
       <c r="E23" s="21" t="n">
-        <v>0.06</v>
+        <v>-0.03</v>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="G23" s="21" t="n">
         <v>0.07</v>
@@ -3603,10 +3603,10 @@
       <c r="C24" s="19"/>
       <c r="D24" s="19"/>
       <c r="E24" s="21" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="F24" s="21" t="n">
         <v>0.04</v>
-      </c>
-      <c r="F24" s="21" t="n">
-        <v>0.05</v>
       </c>
       <c r="G24" s="21" t="n">
         <v>0.06</v>
@@ -3615,7 +3615,7 @@
         <v>0.05</v>
       </c>
       <c r="I24" s="21" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,10 +3626,10 @@
       <c r="C25" s="19"/>
       <c r="D25" s="19"/>
       <c r="E25" s="21" t="n">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G25" s="21" t="n">
         <v>0.06</v>
@@ -3649,10 +3649,10 @@
       <c r="C26" s="19"/>
       <c r="D26" s="19"/>
       <c r="E26" s="21" t="n">
-        <v>0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="F26" s="21" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="G26" s="21" t="n">
         <v>0.07</v>
@@ -3672,13 +3672,13 @@
       <c r="C27" s="19"/>
       <c r="D27" s="19"/>
       <c r="E27" s="21" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="G27" s="21" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="H27" s="21" t="n">
         <v>0.04</v>
@@ -3708,19 +3708,19 @@
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
       <c r="E30" s="21" t="n">
-        <v>0.01</v>
+        <v>-0.09</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="G30" s="21" t="n">
         <v>0.02</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="I30" s="21" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,10 +3731,10 @@
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
       <c r="E31" s="21" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="F31" s="21" t="n">
         <v>-0.02</v>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0</v>
       </c>
       <c r="G31" s="21" t="n">
         <v>0.01</v>
@@ -3754,13 +3754,13 @@
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
       <c r="E32" s="21" t="n">
-        <v>-0.12</v>
+        <v>-0.26</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>-0.06</v>
+        <v>-0.1</v>
       </c>
       <c r="G32" s="21" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="H32" s="21" t="n">
         <v>0</v>
@@ -3777,10 +3777,10 @@
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
       <c r="E33" s="21" t="n">
-        <v>-0.01</v>
+        <v>-0.09</v>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G33" s="21" t="n">
         <v>0.02</v>
@@ -3800,10 +3800,10 @@
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
       <c r="E34" s="21" t="n">
-        <v>-0.18</v>
+        <v>-0.2</v>
       </c>
       <c r="F34" s="21" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="G34" s="21" t="n">
         <v>-0.03</v>
@@ -3859,16 +3859,16 @@
       <c r="C39" s="19"/>
       <c r="D39" s="19"/>
       <c r="E39" s="21" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="F39" s="21" t="n">
         <v>0.43</v>
       </c>
-      <c r="F39" s="21" t="n">
+      <c r="G39" s="21" t="n">
         <v>0.435</v>
       </c>
-      <c r="G39" s="21" t="n">
+      <c r="H39" s="21" t="n">
         <v>0.44</v>
-      </c>
-      <c r="H39" s="21" t="n">
-        <v>0.445</v>
       </c>
       <c r="I39" s="21" t="n">
         <v>0.445</v>
@@ -3882,16 +3882,16 @@
       <c r="C40" s="19"/>
       <c r="D40" s="19"/>
       <c r="E40" s="21" t="n">
-        <v>0.435</v>
+        <v>0.43</v>
       </c>
       <c r="F40" s="21" t="n">
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="G40" s="21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H40" s="21" t="n">
         <v>0.455</v>
-      </c>
-      <c r="H40" s="21" t="n">
-        <v>0.46</v>
       </c>
       <c r="I40" s="21" t="n">
         <v>0.46</v>
@@ -3905,13 +3905,13 @@
       <c r="C41" s="19"/>
       <c r="D41" s="19"/>
       <c r="E41" s="21" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G41" s="21" t="n">
         <v>0.425</v>
-      </c>
-      <c r="F41" s="21" t="n">
-        <v>0.425</v>
-      </c>
-      <c r="G41" s="21" t="n">
-        <v>0.428</v>
       </c>
       <c r="H41" s="21" t="n">
         <v>0.43</v>
@@ -3929,19 +3929,19 @@
       <c r="D42" s="19"/>
       <c r="E42" s="24" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,E39,E40,E41)</f>
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="F42" s="24" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,F39,F40,F41)</f>
-        <v>0.435</v>
+        <v>0.43</v>
       </c>
       <c r="G42" s="24" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,G39,G40,G41)</f>
-        <v>0.44</v>
+        <v>0.435</v>
       </c>
       <c r="H42" s="24" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,H39,H40,H41)</f>
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="I42" s="24" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$6,I39,I40,I41)</f>
@@ -3956,19 +3956,19 @@
       <c r="C43" s="19"/>
       <c r="D43" s="19"/>
       <c r="E43" s="25" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="F43" s="25" t="n">
-        <v>0.098</v>
+        <v>0.102</v>
       </c>
       <c r="G43" s="25" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="H43" s="25" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="I43" s="25" t="n">
         <v>0.096</v>
-      </c>
-      <c r="H43" s="25" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="I43" s="25" t="n">
-        <v>0.095</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3979,19 +3979,19 @@
       <c r="C44" s="19"/>
       <c r="D44" s="19"/>
       <c r="E44" s="25" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="F44" s="25" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G44" s="25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H44" s="25" t="n">
         <v>0.243</v>
       </c>
-      <c r="F44" s="25" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="G44" s="25" t="n">
-        <v>0.237</v>
-      </c>
-      <c r="H44" s="25" t="n">
-        <v>0.235</v>
-      </c>
       <c r="I44" s="25" t="n">
-        <v>0.233</v>
+        <v>0.238</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4317,13 +4317,13 @@
       <c r="C63" s="19"/>
       <c r="D63" s="19"/>
       <c r="E63" s="21" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F63" s="21" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="G63" s="21" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="H63" s="21" t="n">
         <v>0.05</v>
@@ -4340,19 +4340,19 @@
       <c r="C64" s="22"/>
       <c r="D64" s="22"/>
       <c r="E64" s="23" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="F64" s="23" t="n">
-        <v>2000</v>
+        <v>750</v>
       </c>
       <c r="G64" s="23" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H64" s="23" t="n">
         <v>2500</v>
       </c>
-      <c r="H64" s="23" t="n">
+      <c r="I64" s="23" t="n">
         <v>3000</v>
-      </c>
-      <c r="I64" s="23" t="n">
-        <v>3500</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4363,19 +4363,19 @@
       <c r="C65" s="28"/>
       <c r="D65" s="28"/>
       <c r="E65" s="29" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F65" s="29" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="G65" s="29" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="H65" s="29" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="I65" s="29" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4489,23 +4489,23 @@
       </c>
       <c r="E6" s="33" t="n">
         <f aca="false">D6*(1+Assumptions!E9)</f>
-        <v>21331.44</v>
+        <v>19280.34</v>
       </c>
       <c r="F6" s="33" t="n">
         <f aca="false">E6*(1+Assumptions!F9)</f>
-        <v>22398.012</v>
+        <v>19858.7502</v>
       </c>
       <c r="G6" s="33" t="n">
         <f aca="false">F6*(1+Assumptions!G9)</f>
-        <v>23517.9126</v>
+        <v>20851.68771</v>
       </c>
       <c r="H6" s="33" t="n">
         <f aca="false">G6*(1+Assumptions!H9)</f>
-        <v>24458.629104</v>
+        <v>21894.2720955</v>
       </c>
       <c r="I6" s="33" t="n">
         <f aca="false">H6*(1+Assumptions!I9)</f>
-        <v>25436.97426816</v>
+        <v>22770.04297932</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4521,23 +4521,23 @@
       </c>
       <c r="E7" s="33" t="n">
         <f aca="false">D7*(1+Assumptions!E10)</f>
-        <v>12823.44</v>
+        <v>11566.24</v>
       </c>
       <c r="F7" s="33" t="n">
         <f aca="false">E7*(1+Assumptions!F10)</f>
-        <v>13208.1432</v>
+        <v>11797.5648</v>
       </c>
       <c r="G7" s="33" t="n">
         <f aca="false">F7*(1+Assumptions!G10)</f>
-        <v>13736.468928</v>
+        <v>12269.467392</v>
       </c>
       <c r="H7" s="33" t="n">
         <f aca="false">G7*(1+Assumptions!H10)</f>
-        <v>14285.92768512</v>
+        <v>12760.24608768</v>
       </c>
       <c r="I7" s="33" t="n">
         <f aca="false">H7*(1+Assumptions!I10)</f>
-        <v>14714.5055156736</v>
+        <v>13270.6559311872</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4553,23 +4553,23 @@
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">D8*(1+Assumptions!E11)</f>
-        <v>5554.65</v>
+        <v>4677.6</v>
       </c>
       <c r="F8" s="33" t="n">
         <f aca="false">E8*(1+Assumptions!F11)</f>
-        <v>5554.65</v>
+        <v>4537.272</v>
       </c>
       <c r="G8" s="33" t="n">
         <f aca="false">F8*(1+Assumptions!G11)</f>
-        <v>5721.2895</v>
+        <v>4673.39016</v>
       </c>
       <c r="H8" s="33" t="n">
         <f aca="false">G8*(1+Assumptions!H11)</f>
-        <v>5950.14108</v>
+        <v>4860.3257664</v>
       </c>
       <c r="I8" s="33" t="n">
         <f aca="false">H8*(1+Assumptions!I11)</f>
-        <v>6188.1467232</v>
+        <v>5054.738797056</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4585,23 +4585,23 @@
       </c>
       <c r="E9" s="33" t="n">
         <f aca="false">D9*(1+Assumptions!E12)</f>
-        <v>6367.86</v>
+        <v>5868.42</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">E9*(1+Assumptions!F12)</f>
-        <v>6622.5744</v>
+        <v>6044.4726</v>
       </c>
       <c r="G9" s="33" t="n">
         <f aca="false">F9*(1+Assumptions!G12)</f>
-        <v>6953.70312</v>
+        <v>6346.69623</v>
       </c>
       <c r="H9" s="33" t="n">
         <f aca="false">G9*(1+Assumptions!H12)</f>
-        <v>7301.388276</v>
+        <v>6664.0310415</v>
       </c>
       <c r="I9" s="33" t="n">
         <f aca="false">H9*(1+Assumptions!I12)</f>
-        <v>7666.4576898</v>
+        <v>6997.232593575</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4617,23 +4617,23 @@
       </c>
       <c r="E10" s="33" t="n">
         <f aca="false">D10*(1+Assumptions!E13)</f>
-        <v>1056.6</v>
+        <v>997.9</v>
       </c>
       <c r="F10" s="33" t="n">
         <f aca="false">E10*(1+Assumptions!F13)</f>
-        <v>1024.902</v>
+        <v>948.005</v>
       </c>
       <c r="G10" s="33" t="n">
         <f aca="false">F10*(1+Assumptions!G13)</f>
-        <v>1045.40004</v>
+        <v>948.005</v>
       </c>
       <c r="H10" s="33" t="n">
         <f aca="false">G10*(1+Assumptions!H13)</f>
-        <v>1066.3080408</v>
+        <v>966.9651</v>
       </c>
       <c r="I10" s="33" t="n">
         <f aca="false">H10*(1+Assumptions!I13)</f>
-        <v>1087.634201616</v>
+        <v>986.304402</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4685,23 +4685,23 @@
       </c>
       <c r="E12" s="36" t="n">
         <f aca="false">SUM(E6:E11)</f>
-        <v>47184.99</v>
+        <v>42441.5</v>
       </c>
       <c r="F12" s="36" t="n">
         <f aca="false">SUM(F6:F11)</f>
-        <v>48859.2816</v>
+        <v>43237.0646</v>
       </c>
       <c r="G12" s="36" t="n">
         <f aca="false">SUM(G6:G11)</f>
-        <v>51025.774188</v>
+        <v>45140.246492</v>
       </c>
       <c r="H12" s="36" t="n">
         <f aca="false">SUM(H6:H11)</f>
-        <v>53113.39418592</v>
+        <v>47196.84009108</v>
       </c>
       <c r="I12" s="36" t="n">
         <f aca="false">SUM(I6:I11)</f>
-        <v>55144.7183984496</v>
+        <v>49129.9747031382</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4729,11 +4729,11 @@
       </c>
       <c r="E15" s="37" t="n">
         <f aca="false">E6/D6-1</f>
-        <v>0.04</v>
+        <v>-0.0599999999999999</v>
       </c>
       <c r="F15" s="37" t="n">
         <f aca="false">F6/E6-1</f>
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G15" s="37" t="n">
         <f aca="false">G6/F6-1</f>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="H15" s="37" t="n">
         <f aca="false">H6/G6-1</f>
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="I15" s="37" t="n">
         <f aca="false">I6/H6-1</f>
@@ -4760,11 +4760,11 @@
       </c>
       <c r="E16" s="37" t="n">
         <f aca="false">E7/D7-1</f>
-        <v>0.02</v>
+        <v>-0.0800000000000001</v>
       </c>
       <c r="F16" s="37" t="n">
         <f aca="false">F7/E7-1</f>
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="G16" s="37" t="n">
         <f aca="false">G7/F7-1</f>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="I16" s="37" t="n">
         <f aca="false">I7/H7-1</f>
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4791,11 +4791,11 @@
       </c>
       <c r="E17" s="37" t="n">
         <f aca="false">E8/D8-1</f>
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="F17" s="37" t="n">
         <f aca="false">F8/E8-1</f>
-        <v>0</v>
+        <v>-0.0300000000000001</v>
       </c>
       <c r="G17" s="37" t="n">
         <f aca="false">G8/F8-1</f>
@@ -4822,11 +4822,11 @@
       </c>
       <c r="E18" s="37" t="n">
         <f aca="false">E9/D9-1</f>
-        <v>0.02</v>
+        <v>-0.0599999999999999</v>
       </c>
       <c r="F18" s="37" t="n">
         <f aca="false">F9/E9-1</f>
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="G18" s="37" t="n">
         <f aca="false">G9/F9-1</f>
@@ -4853,15 +4853,15 @@
       </c>
       <c r="E19" s="37" t="n">
         <f aca="false">E10/D10-1</f>
-        <v>-0.0999999999999999</v>
+        <v>-0.15</v>
       </c>
       <c r="F19" s="37" t="n">
         <f aca="false">F10/E10-1</f>
-        <v>-0.0300000000000001</v>
+        <v>-0.05</v>
       </c>
       <c r="G19" s="37" t="n">
         <f aca="false">G10/F10-1</f>
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H19" s="37" t="n">
         <f aca="false">H10/G10-1</f>
@@ -4887,23 +4887,23 @@
       </c>
       <c r="E20" s="20" t="n">
         <f aca="false">E12/D12-1</f>
-        <v>0.0169617224880383</v>
+        <v>-0.0852730721151774</v>
       </c>
       <c r="F20" s="20" t="n">
         <f aca="false">F12/E12-1</f>
-        <v>0.0354835637349928</v>
+        <v>0.0187449689572707</v>
       </c>
       <c r="G20" s="20" t="n">
         <f aca="false">G12/F12-1</f>
-        <v>0.0443414744763664</v>
+        <v>0.0440173705039171</v>
       </c>
       <c r="H20" s="20" t="n">
         <f aca="false">H12/G12-1</f>
-        <v>0.0409130489667506</v>
+        <v>0.0455600879238549</v>
       </c>
       <c r="I20" s="20" t="n">
         <f aca="false">I12/H12-1</f>
-        <v>0.0382450461632913</v>
+        <v>0.0409589838711164</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4934,23 +4934,23 @@
       </c>
       <c r="E23" s="37" t="n">
         <f aca="false">E6/E12</f>
-        <v>0.452081053741879</v>
+        <v>0.45428036238116</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">F6/F12</f>
-        <v>0.458418774622343</v>
+        <v>0.459299223564775</v>
       </c>
       <c r="G23" s="37" t="n">
         <f aca="false">G6/G12</f>
-        <v>0.460902611949606</v>
+        <v>0.461931188472696</v>
       </c>
       <c r="H23" s="37" t="n">
         <f aca="false">H6/H12</f>
-        <v>0.46049832587208</v>
+        <v>0.463892753270106</v>
       </c>
       <c r="I23" s="37" t="n">
         <f aca="false">I6/I12</f>
-        <v>0.461276709844894</v>
+        <v>0.46346539188968</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4968,23 +4968,23 @@
       </c>
       <c r="E24" s="37" t="n">
         <f aca="false">E7/E12</f>
-        <v>0.271769475843907</v>
+        <v>0.272521941967178</v>
       </c>
       <c r="F24" s="37" t="n">
         <f aca="false">F7/F12</f>
-        <v>0.270330278454197</v>
+        <v>0.27285767221117</v>
       </c>
       <c r="G24" s="37" t="n">
         <f aca="false">G7/G12</f>
-        <v>0.269206477443913</v>
+        <v>0.271807718067611</v>
       </c>
       <c r="H24" s="37" t="n">
         <f aca="false">H7/H12</f>
-        <v>0.268970339856516</v>
+        <v>0.270362296777823</v>
       </c>
       <c r="I24" s="37" t="n">
         <f aca="false">I7/I12</f>
-        <v>0.266834357723138</v>
+        <v>0.27011322540615</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5002,23 +5002,23 @@
       </c>
       <c r="E25" s="37" t="n">
         <f aca="false">E8/E12</f>
-        <v>0.117720698891745</v>
+        <v>0.110212881260087</v>
       </c>
       <c r="F25" s="37" t="n">
         <f aca="false">F8/F12</f>
-        <v>0.11368668998195</v>
+        <v>0.104939408860795</v>
       </c>
       <c r="G25" s="37" t="n">
         <f aca="false">G8/G12</f>
-        <v>0.1121254815051</v>
+        <v>0.103530452826133</v>
       </c>
       <c r="H25" s="37" t="n">
         <f aca="false">H8/H12</f>
-        <v>0.112027129337129</v>
+        <v>0.10297989774359</v>
       </c>
       <c r="I25" s="37" t="n">
         <f aca="false">I8/I12</f>
-        <v>0.112216489682428</v>
+        <v>0.102885027472508</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5036,23 +5036,23 @@
       </c>
       <c r="E26" s="37" t="n">
         <f aca="false">E9/E12</f>
-        <v>0.134955205034482</v>
+        <v>0.138270796272516</v>
       </c>
       <c r="F26" s="37" t="n">
         <f aca="false">F9/F12</f>
-        <v>0.13554383493023</v>
+        <v>0.139798403428155</v>
       </c>
       <c r="G26" s="37" t="n">
         <f aca="false">G9/G12</f>
-        <v>0.136278248211966</v>
+        <v>0.140599503175615</v>
       </c>
       <c r="H26" s="37" t="n">
         <f aca="false">H9/H12</f>
-        <v>0.137467928531209</v>
+        <v>0.141196551053838</v>
       </c>
       <c r="I26" s="37" t="n">
         <f aca="false">I9/I12</f>
-        <v>0.13902433292715</v>
+        <v>0.142422882076673</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5070,23 +5070,23 @@
       </c>
       <c r="E27" s="37" t="n">
         <f aca="false">E10/E12</f>
-        <v>0.022392714293253</v>
+        <v>0.0235123640776127</v>
       </c>
       <c r="F27" s="37" t="n">
         <f aca="false">F10/F12</f>
-        <v>0.0209766080555716</v>
+        <v>0.0219257484005979</v>
       </c>
       <c r="G27" s="37" t="n">
         <f aca="false">G10/G12</f>
-        <v>0.0204876860103742</v>
+        <v>0.0210013252844778</v>
       </c>
       <c r="H27" s="37" t="n">
         <f aca="false">H10/H12</f>
-        <v>0.0200760666333516</v>
+        <v>0.0204879203381828</v>
       </c>
       <c r="I27" s="37" t="n">
         <f aca="false">I10/I12</f>
-        <v>0.0197232705724829</v>
+        <v>0.0200754103367572</v>
       </c>
     </row>
   </sheetData>
@@ -5166,23 +5166,23 @@
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">'Revenue Build'!E12</f>
-        <v>47184.99</v>
+        <v>42441.5</v>
       </c>
       <c r="F5" s="10" t="n">
         <f aca="false">'Revenue Build'!F12</f>
-        <v>48859.2816</v>
+        <v>43237.0646</v>
       </c>
       <c r="G5" s="10" t="n">
         <f aca="false">'Revenue Build'!G12</f>
-        <v>51025.774188</v>
+        <v>45140.246492</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">'Revenue Build'!H12</f>
-        <v>53113.39418592</v>
+        <v>47196.84009108</v>
       </c>
       <c r="I5" s="10" t="n">
         <f aca="false">'Revenue Build'!I12</f>
-        <v>55144.7183984496</v>
+        <v>49129.9747031382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5200,23 +5200,23 @@
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">E5*(1-Assumptions!E42)</f>
-        <v>26895.4443</v>
+        <v>24403.8625</v>
       </c>
       <c r="F6" s="10" t="n">
         <f aca="false">F5*(1-Assumptions!F42)</f>
-        <v>27605.494104</v>
+        <v>24645.126822</v>
       </c>
       <c r="G6" s="10" t="n">
         <f aca="false">G5*(1-Assumptions!G42)</f>
-        <v>28574.43354528</v>
+        <v>25504.23926798</v>
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">H5*(1-Assumptions!H42)</f>
-        <v>29477.9337731856</v>
+        <v>26430.2304510048</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">I5*(1-Assumptions!I42)</f>
-        <v>30605.3187111395</v>
+        <v>27267.1359602417</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5237,23 +5237,23 @@
       </c>
       <c r="E7" s="36" t="n">
         <f aca="false">E5-E6</f>
-        <v>20289.5457</v>
+        <v>18037.6375</v>
       </c>
       <c r="F7" s="36" t="n">
         <f aca="false">F5-F6</f>
-        <v>21253.787496</v>
+        <v>18591.937778</v>
       </c>
       <c r="G7" s="36" t="n">
         <f aca="false">G5-G6</f>
-        <v>22451.34064272</v>
+        <v>19636.00722402</v>
       </c>
       <c r="H7" s="36" t="n">
         <f aca="false">H5-H6</f>
-        <v>23635.4604127344</v>
+        <v>20766.6096400752</v>
       </c>
       <c r="I7" s="36" t="n">
         <f aca="false">I5-I6</f>
-        <v>24539.3996873101</v>
+        <v>21862.8387428965</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5271,23 +5271,23 @@
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">E5*Assumptions!E43</f>
-        <v>4718.499</v>
+        <v>4456.3575</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">F5*Assumptions!F43</f>
-        <v>4788.2095968</v>
+        <v>4410.1805892</v>
       </c>
       <c r="G8" s="10" t="n">
         <f aca="false">G5*Assumptions!G43</f>
-        <v>4898.474322048</v>
+        <v>4468.884402708</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">H5*Assumptions!H43</f>
-        <v>5045.7724476624</v>
+        <v>4578.09348883476</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">I5*Assumptions!I43</f>
-        <v>5238.74824785271</v>
+        <v>4716.47757150127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5305,23 +5305,23 @@
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">E5*Assumptions!E44</f>
-        <v>11465.95257</v>
+        <v>11586.5295</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">F5*Assumptions!F44</f>
-        <v>11726.227584</v>
+        <v>11241.636796</v>
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">G5*Assumptions!G44</f>
-        <v>12093.108482556</v>
+        <v>11285.061623</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">H5*Assumptions!H44</f>
-        <v>12481.6476336912</v>
+        <v>11468.8321421324</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">I5*Assumptions!I44</f>
-        <v>12848.7193868388</v>
+        <v>11692.9339793469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5342,23 +5342,23 @@
       </c>
       <c r="E10" s="36" t="n">
         <f aca="false">E7-E8-E9</f>
-        <v>4105.09413</v>
+        <v>1994.7505</v>
       </c>
       <c r="F10" s="36" t="n">
         <f aca="false">F7-F8-F9</f>
-        <v>4739.35031520001</v>
+        <v>2940.1203928</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">G7-G8-G9</f>
-        <v>5459.757838116</v>
+        <v>3882.061198312</v>
       </c>
       <c r="H10" s="36" t="n">
         <f aca="false">H7-H8-H9</f>
-        <v>6108.04033138081</v>
+        <v>4719.684009108</v>
       </c>
       <c r="I10" s="36" t="n">
         <f aca="false">I7-I8-I9</f>
-        <v>6451.93205261861</v>
+        <v>5453.42719204834</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5380,19 +5380,19 @@
       </c>
       <c r="F11" s="10" t="n">
         <f aca="false">Assumptions!F51*('Balance Sheet'!E19+'Balance Sheet'!E25)-Assumptions!F52*('Balance Sheet'!E6+'Balance Sheet'!E7)</f>
-        <v>-44.5113600052251</v>
+        <v>-30.0846258852314</v>
       </c>
       <c r="G11" s="10" t="n">
         <f aca="false">Assumptions!G51*('Balance Sheet'!F19+'Balance Sheet'!F25)-Assumptions!G52*('Balance Sheet'!F6+'Balance Sheet'!F7)</f>
-        <v>-53.5870080775806</v>
+        <v>-37.7597754707801</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">Assumptions!H51*('Balance Sheet'!G19+'Balance Sheet'!G25)-Assumptions!H52*('Balance Sheet'!G6+'Balance Sheet'!G7)</f>
-        <v>-63.4293630637411</v>
+        <v>-42.5983010697049</v>
       </c>
       <c r="I11" s="10" t="n">
         <f aca="false">Assumptions!I51*('Balance Sheet'!H19+'Balance Sheet'!H25)-Assumptions!I52*('Balance Sheet'!H6+'Balance Sheet'!H7)</f>
-        <v>-61.5430510000264</v>
+        <v>-24.5394865938578</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>107</v>
@@ -5448,23 +5448,23 @@
       </c>
       <c r="E13" s="36" t="n">
         <f aca="false">E10-E11-E12</f>
-        <v>4103.35913</v>
+        <v>1993.0155</v>
       </c>
       <c r="F13" s="36" t="n">
         <f aca="false">F10-F11-F12</f>
-        <v>4783.86167520523</v>
+        <v>2970.20501868523</v>
       </c>
       <c r="G13" s="36" t="n">
         <f aca="false">G10-G11-G12</f>
-        <v>5513.34484619358</v>
+        <v>3919.82097378278</v>
       </c>
       <c r="H13" s="36" t="n">
         <f aca="false">H10-H11-H12</f>
-        <v>6171.46969444455</v>
+        <v>4762.2823101777</v>
       </c>
       <c r="I13" s="36" t="n">
         <f aca="false">I10-I11-I12</f>
-        <v>6513.47510361864</v>
+        <v>5477.9666786422</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5482,23 +5482,23 @@
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">E13*Assumptions!E50</f>
-        <v>779.6382347</v>
+        <v>378.672945</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">F13*Assumptions!F50</f>
-        <v>908.933718288994</v>
+        <v>564.338953550193</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">G13*Assumptions!G50</f>
-        <v>1047.53552077678</v>
+        <v>744.765985018729</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">H13*Assumptions!H50</f>
-        <v>1172.57924194446</v>
+        <v>904.833638933763</v>
       </c>
       <c r="I14" s="10" t="n">
         <f aca="false">I13*Assumptions!I50</f>
-        <v>1237.56026968754</v>
+        <v>1040.81366894202</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5519,23 +5519,23 @@
       </c>
       <c r="E15" s="40" t="n">
         <f aca="false">E13-E14</f>
-        <v>3323.7208953</v>
+        <v>1614.342555</v>
       </c>
       <c r="F15" s="40" t="n">
         <f aca="false">F13-F14</f>
-        <v>3874.92795691624</v>
+        <v>2405.86606513503</v>
       </c>
       <c r="G15" s="40" t="n">
         <f aca="false">G13-G14</f>
-        <v>4465.8093254168</v>
+        <v>3175.05498876406</v>
       </c>
       <c r="H15" s="40" t="n">
         <f aca="false">H13-H14</f>
-        <v>4998.89045250008</v>
+        <v>3857.44867124394</v>
       </c>
       <c r="I15" s="40" t="n">
         <f aca="false">I13-I14</f>
-        <v>5275.91483393109</v>
+        <v>4437.15300970018</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5553,23 +5553,23 @@
       </c>
       <c r="E17" s="42" t="n">
         <f aca="false">D17-Assumptions!E64/Assumptions!E65+Assumptions!E66</f>
-        <v>1475.66666666667</v>
+        <v>1482.75</v>
       </c>
       <c r="F17" s="42" t="n">
         <f aca="false">E17-Assumptions!F64/Assumptions!F65+Assumptions!F66</f>
-        <v>1457</v>
+        <v>1474.08333333333</v>
       </c>
       <c r="G17" s="42" t="n">
         <f aca="false">F17-Assumptions!G64/Assumptions!G65+Assumptions!G66</f>
-        <v>1431.66666666667</v>
+        <v>1452.08333333333</v>
       </c>
       <c r="H17" s="42" t="n">
         <f aca="false">G17-Assumptions!H64/Assumptions!H65+Assumptions!H66</f>
-        <v>1399.66666666667</v>
+        <v>1414.62878787879</v>
       </c>
       <c r="I17" s="42" t="n">
         <f aca="false">H17-Assumptions!I64/Assumptions!I65+Assumptions!I66</f>
-        <v>1361</v>
+        <v>1372.62878787879</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5590,23 +5590,23 @@
       </c>
       <c r="E18" s="44" t="n">
         <f aca="false">E15/E17</f>
-        <v>2.25235208626609</v>
+        <v>1.08874898330804</v>
       </c>
       <c r="F18" s="44" t="n">
         <f aca="false">F15/F17</f>
-        <v>2.65952502190545</v>
+        <v>1.63210994299397</v>
       </c>
       <c r="G18" s="44" t="n">
         <f aca="false">G15/G17</f>
-        <v>3.11930802706645</v>
+        <v>2.18655149871843</v>
       </c>
       <c r="H18" s="44" t="n">
         <f aca="false">H15/H17</f>
-        <v>3.57148639140278</v>
+        <v>2.72682749304722</v>
       </c>
       <c r="I18" s="44" t="n">
         <f aca="false">I15/I17</f>
-        <v>3.87649877584944</v>
+        <v>3.23259503871925</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5627,23 +5627,23 @@
       </c>
       <c r="E19" s="14" t="n">
         <f aca="false">D19*(1+Assumptions!E63)</f>
-        <v>1.70651586765699</v>
+        <v>1.62525320729237</v>
       </c>
       <c r="F19" s="14" t="n">
         <f aca="false">E19*(1+Assumptions!F63)</f>
-        <v>1.79184166103984</v>
+        <v>1.62525320729237</v>
       </c>
       <c r="G19" s="14" t="n">
         <f aca="false">F19*(1+Assumptions!G63)</f>
-        <v>1.88143374409183</v>
+        <v>1.67401080351114</v>
       </c>
       <c r="H19" s="14" t="n">
         <f aca="false">G19*(1+Assumptions!H63)</f>
-        <v>1.97550543129642</v>
+        <v>1.7577113436867</v>
       </c>
       <c r="I19" s="14" t="n">
         <f aca="false">H19*(1+Assumptions!I63)</f>
-        <v>2.07428070286124</v>
+        <v>1.84559691087103</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5677,19 +5677,19 @@
       </c>
       <c r="E22" s="37" t="n">
         <f aca="false">E7/E5</f>
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="F22" s="37" t="n">
         <f aca="false">F7/F5</f>
-        <v>0.435</v>
+        <v>0.43</v>
       </c>
       <c r="G22" s="37" t="n">
         <f aca="false">G7/G5</f>
-        <v>0.44</v>
+        <v>0.435</v>
       </c>
       <c r="H22" s="37" t="n">
         <f aca="false">H7/H5</f>
-        <v>0.445</v>
+        <v>0.44</v>
       </c>
       <c r="I22" s="37" t="n">
         <f aca="false">I7/I5</f>
@@ -5714,23 +5714,23 @@
       </c>
       <c r="E23" s="37" t="n">
         <f aca="false">E8/E5</f>
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">F8/F5</f>
-        <v>0.098</v>
+        <v>0.102</v>
       </c>
       <c r="G23" s="37" t="n">
         <f aca="false">G8/G5</f>
-        <v>0.096</v>
+        <v>0.099</v>
       </c>
       <c r="H23" s="37" t="n">
         <f aca="false">H8/H5</f>
-        <v>0.095</v>
+        <v>0.097</v>
       </c>
       <c r="I23" s="37" t="n">
         <f aca="false">I8/I5</f>
-        <v>0.095</v>
+        <v>0.096</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5751,23 +5751,23 @@
       </c>
       <c r="E24" s="37" t="n">
         <f aca="false">E9/E5</f>
-        <v>0.243</v>
+        <v>0.273</v>
       </c>
       <c r="F24" s="37" t="n">
         <f aca="false">F9/F5</f>
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="G24" s="37" t="n">
         <f aca="false">G9/G5</f>
-        <v>0.237</v>
+        <v>0.25</v>
       </c>
       <c r="H24" s="37" t="n">
         <f aca="false">H9/H5</f>
-        <v>0.235</v>
+        <v>0.243</v>
       </c>
       <c r="I24" s="37" t="n">
         <f aca="false">I9/I5</f>
-        <v>0.233</v>
+        <v>0.238</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5788,23 +5788,23 @@
       </c>
       <c r="E25" s="37" t="n">
         <f aca="false">E10/E5</f>
-        <v>0.0869999999999999</v>
+        <v>0.047</v>
       </c>
       <c r="F25" s="37" t="n">
         <f aca="false">F10/F5</f>
-        <v>0.0970000000000001</v>
+        <v>0.0679999999999999</v>
       </c>
       <c r="G25" s="37" t="n">
         <f aca="false">G10/G5</f>
-        <v>0.107</v>
+        <v>0.0860000000000001</v>
       </c>
       <c r="H25" s="37" t="n">
         <f aca="false">H10/H5</f>
-        <v>0.115</v>
+        <v>0.0999999999999999</v>
       </c>
       <c r="I25" s="37" t="n">
         <f aca="false">I10/I5</f>
-        <v>0.117</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5825,23 +5825,23 @@
       </c>
       <c r="E26" s="37" t="n">
         <f aca="false">E15/E5</f>
-        <v>0.0704402161640809</v>
+        <v>0.038036887362605</v>
       </c>
       <c r="F26" s="37" t="n">
         <f aca="false">F15/F5</f>
-        <v>0.0793079191920873</v>
+        <v>0.0556436031768686</v>
       </c>
       <c r="G26" s="37" t="n">
         <f aca="false">G15/G5</f>
-        <v>0.0875206578730763</v>
+        <v>0.0703375642693213</v>
       </c>
       <c r="H26" s="37" t="n">
         <f aca="false">H15/H5</f>
-        <v>0.0941173225533618</v>
+        <v>0.0817310791103784</v>
       </c>
       <c r="I26" s="37" t="n">
         <f aca="false">I15/I5</f>
-        <v>0.0956739826978503</v>
+        <v>0.0903145795720663</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5971,23 +5971,23 @@
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">'Cash Flow'!E32</f>
-        <v>6598.61028586357</v>
+        <v>6186.41788243518</v>
       </c>
       <c r="F6" s="10" t="n">
         <f aca="false">'Cash Flow'!F32</f>
-        <v>6857.9145165023</v>
+        <v>6405.70787059372</v>
       </c>
       <c r="G6" s="10" t="n">
         <f aca="false">'Cash Flow'!G32</f>
-        <v>7139.12465896403</v>
+        <v>6543.95145913443</v>
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">'Cash Flow'!H32</f>
-        <v>7085.23002857218</v>
+        <v>6027.98533125308</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">'Cash Flow'!I32</f>
-        <v>6676.27862376154</v>
+        <v>5518.05445312302</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6039,23 +6039,23 @@
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">'Income Statement'!E5*Assumptions!E55/365</f>
-        <v>5688.0535890411</v>
+        <v>5116.23561643836</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">'Income Statement'!F5*Assumptions!F55/365</f>
-        <v>5622.16391013699</v>
+        <v>4975.22387178082</v>
       </c>
       <c r="G8" s="10" t="n">
         <f aca="false">'Income Statement'!G5*Assumptions!G55/365</f>
-        <v>5591.86566443836</v>
+        <v>4946.87632789041</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">'Income Statement'!H5*Assumptions!H55/365</f>
-        <v>5820.64593818301</v>
+        <v>5172.25644833753</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">'Income Statement'!I5*Assumptions!I55/365</f>
-        <v>6043.256810789</v>
+        <v>5384.10681678227</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6073,23 +6073,23 @@
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">'Income Statement'!E6*Assumptions!E56/365</f>
-        <v>7368.61487671233</v>
+        <v>6685.9897260274</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">'Income Statement'!F6*Assumptions!F56/365</f>
-        <v>7411.88608819726</v>
+        <v>6617.04774946849</v>
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">'Income Statement'!G6*Assumptions!G56/365</f>
-        <v>7515.46745300515</v>
+        <v>6707.9643006194</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">'Income Statement'!H6*Assumptions!H56/365</f>
-        <v>7672.33892726748</v>
+        <v>6879.10107628892</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">'Income Statement'!I6*Assumptions!I56/365</f>
-        <v>7965.76788372125</v>
+        <v>7096.92579787113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6107,23 +6107,23 @@
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">'Income Statement'!E5*Assumptions!E58</f>
-        <v>2170.50954</v>
+        <v>1952.309</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">'Income Statement'!F5*Assumptions!F58</f>
-        <v>2247.5269536</v>
+        <v>1988.9049716</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">'Income Statement'!G5*Assumptions!G58</f>
-        <v>2347.185612648</v>
+        <v>2076.451338632</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">'Income Statement'!H5*Assumptions!H58</f>
-        <v>2443.21613255232</v>
+        <v>2171.05464418968</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">'Income Statement'!I5*Assumptions!I58</f>
-        <v>2536.65704632868</v>
+        <v>2259.97883634436</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6144,23 +6144,23 @@
       </c>
       <c r="E11" s="36" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>23289.788291617</v>
+        <v>21404.9522249009</v>
       </c>
       <c r="F11" s="36" t="n">
         <f aca="false">SUM(F6:F10)</f>
-        <v>23603.4914684366</v>
+        <v>21450.884463443</v>
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">SUM(G6:G10)</f>
-        <v>24057.6433890555</v>
+        <v>21739.2434262762</v>
       </c>
       <c r="H11" s="36" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>24485.431026575</v>
+        <v>21714.3975000692</v>
       </c>
       <c r="I11" s="36" t="n">
         <f aca="false">SUM(I6:I10)</f>
-        <v>24685.9603646005</v>
+        <v>21723.0659041208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6317,23 +6317,23 @@
       </c>
       <c r="E16" s="40" t="n">
         <f aca="false">E11+SUM(E12:E15)</f>
-        <v>37096.788291617</v>
+        <v>35211.9522249009</v>
       </c>
       <c r="F16" s="40" t="n">
         <f aca="false">F11+SUM(F12:F15)</f>
-        <v>37410.4914684366</v>
+        <v>35257.884463443</v>
       </c>
       <c r="G16" s="40" t="n">
         <f aca="false">G11+SUM(G12:G15)</f>
-        <v>37864.6433890555</v>
+        <v>35546.2434262762</v>
       </c>
       <c r="H16" s="40" t="n">
         <f aca="false">H11+SUM(H12:H15)</f>
-        <v>38292.431026575</v>
+        <v>35521.3975000692</v>
       </c>
       <c r="I16" s="40" t="n">
         <f aca="false">I11+SUM(I12:I15)</f>
-        <v>38492.9603646005</v>
+        <v>35530.0659041208</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6398,23 +6398,23 @@
       </c>
       <c r="E20" s="10" t="n">
         <f aca="false">'Income Statement'!E6*Assumptions!E57/365</f>
-        <v>3684.30743835617</v>
+        <v>3342.9948630137</v>
       </c>
       <c r="F20" s="10" t="n">
         <f aca="false">'Income Statement'!F6*Assumptions!F57/365</f>
-        <v>3781.57453479452</v>
+        <v>3376.04477013699</v>
       </c>
       <c r="G20" s="10" t="n">
         <f aca="false">'Income Statement'!G6*Assumptions!G57/365</f>
-        <v>3914.30596510685</v>
+        <v>3493.7314065726</v>
       </c>
       <c r="H20" s="10" t="n">
         <f aca="false">'Income Statement'!H6*Assumptions!H57/365</f>
-        <v>4038.07311961447</v>
+        <v>3620.57951383627</v>
       </c>
       <c r="I20" s="10" t="n">
         <f aca="false">'Income Statement'!I6*Assumptions!I57/365</f>
-        <v>4192.50941248487</v>
+        <v>3735.2241041427</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6432,23 +6432,23 @@
       </c>
       <c r="E21" s="10" t="n">
         <f aca="false">'Income Statement'!E5*Assumptions!E59</f>
-        <v>6181.23369</v>
+        <v>5559.8365</v>
       </c>
       <c r="F21" s="10" t="n">
         <f aca="false">'Income Statement'!F5*Assumptions!F59</f>
-        <v>6400.5658896</v>
+        <v>5664.0554626</v>
       </c>
       <c r="G21" s="10" t="n">
         <f aca="false">'Income Statement'!G5*Assumptions!G59</f>
-        <v>6684.376418628</v>
+        <v>5913.372290452</v>
       </c>
       <c r="H21" s="10" t="n">
         <f aca="false">'Income Statement'!H5*Assumptions!H59</f>
-        <v>6957.85463835552</v>
+        <v>6182.78605193148</v>
       </c>
       <c r="I21" s="10" t="n">
         <f aca="false">'Income Statement'!I5*Assumptions!I59</f>
-        <v>7223.9581101969</v>
+        <v>6436.02668611111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6537,23 +6537,23 @@
       </c>
       <c r="E24" s="36" t="n">
         <f aca="false">SUM(E19:E23)</f>
-        <v>10720.5411283562</v>
+        <v>9757.8313630137</v>
       </c>
       <c r="F24" s="36" t="n">
         <f aca="false">SUM(F19:F23)</f>
-        <v>11037.1404243945</v>
+        <v>9895.10023273699</v>
       </c>
       <c r="G24" s="36" t="n">
         <f aca="false">SUM(G19:G23)</f>
-        <v>11453.6823837349</v>
+        <v>10262.1036970246</v>
       </c>
       <c r="H24" s="36" t="n">
         <f aca="false">SUM(H19:H23)</f>
-        <v>11850.92775797</v>
+        <v>10658.3655657678</v>
       </c>
       <c r="I24" s="36" t="n">
         <f aca="false">SUM(I19:I23)</f>
-        <v>12271.4675226818</v>
+        <v>11026.2507902538</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6676,23 +6676,23 @@
       </c>
       <c r="E28" s="36" t="n">
         <f aca="false">E24+SUM(E25:E27)</f>
-        <v>21718.5411283562</v>
+        <v>20755.8313630137</v>
       </c>
       <c r="F28" s="36" t="n">
         <f aca="false">F24+SUM(F25:F27)</f>
-        <v>22035.1404243945</v>
+        <v>20893.100232737</v>
       </c>
       <c r="G28" s="36" t="n">
         <f aca="false">G24+SUM(G25:G27)</f>
-        <v>22451.6823837349</v>
+        <v>21260.1036970246</v>
       </c>
       <c r="H28" s="36" t="n">
         <f aca="false">H24+SUM(H25:H27)</f>
-        <v>22848.92775797</v>
+        <v>21656.3655657678</v>
       </c>
       <c r="I28" s="36" t="n">
         <f aca="false">I24+SUM(I25:I27)</f>
-        <v>23269.4675226818</v>
+        <v>22024.2507902538</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6723,23 +6723,23 @@
       </c>
       <c r="E31" s="10" t="n">
         <f aca="false">D31+'Cash Flow'!E8</f>
-        <v>15868.77485</v>
+        <v>15797.6225</v>
       </c>
       <c r="F31" s="10" t="n">
         <f aca="false">E31+'Cash Flow'!F8</f>
-        <v>16601.664074</v>
+        <v>16446.178469</v>
       </c>
       <c r="G31" s="10" t="n">
         <f aca="false">F31+'Cash Flow'!G8</f>
-        <v>17367.05068682</v>
+        <v>17123.28216638</v>
       </c>
       <c r="H31" s="10" t="n">
         <f aca="false">G31+'Cash Flow'!H8</f>
-        <v>18163.7515996088</v>
+        <v>17831.2347677462</v>
       </c>
       <c r="I31" s="10" t="n">
         <f aca="false">H31+'Cash Flow'!I8</f>
-        <v>18990.9223755855</v>
+        <v>18568.1843882933</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6791,23 +6791,23 @@
       </c>
       <c r="E33" s="10" t="n">
         <f aca="false">D33+'Income Statement'!E15+'Cash Flow'!E24+'Cash Flow'!E25</f>
-        <v>-349.527686739165</v>
+        <v>-1200.50163811276</v>
       </c>
       <c r="F33" s="10" t="n">
         <f aca="false">E33+'Income Statement'!F15+'Cash Flow'!F24+'Cash Flow'!F25</f>
-        <v>-1085.31302995797</v>
+        <v>-1940.39423829396</v>
       </c>
       <c r="G33" s="10" t="n">
         <f aca="false">F33+'Income Statement'!G15+'Cash Flow'!G24+'Cash Flow'!G25</f>
-        <v>-1813.08968149931</v>
+        <v>-2696.14243712837</v>
       </c>
       <c r="H33" s="10" t="n">
         <f aca="false">G33+'Income Statement'!H15+'Cash Flow'!H24+'Cash Flow'!H25</f>
-        <v>-2579.24833100379</v>
+        <v>-3825.20283344474</v>
       </c>
       <c r="I33" s="10" t="n">
         <f aca="false">H33+'Income Statement'!I15+'Cash Flow'!I24+'Cash Flow'!I25</f>
-        <v>-3626.42953366684</v>
+        <v>-4921.3692744263</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6828,23 +6828,23 @@
       </c>
       <c r="E34" s="36" t="n">
         <f aca="false">SUM(E31:E33)</f>
-        <v>15378.2471632608</v>
+        <v>14456.1208618872</v>
       </c>
       <c r="F34" s="36" t="n">
         <f aca="false">SUM(F31:F33)</f>
-        <v>15375.351044042</v>
+        <v>14364.784230706</v>
       </c>
       <c r="G34" s="36" t="n">
         <f aca="false">SUM(G31:G33)</f>
-        <v>15412.9610053207</v>
+        <v>14286.1397292516</v>
       </c>
       <c r="H34" s="36" t="n">
         <f aca="false">SUM(H31:H33)</f>
-        <v>15443.503268605</v>
+        <v>13865.0319343015</v>
       </c>
       <c r="I34" s="36" t="n">
         <f aca="false">SUM(I31:I33)</f>
-        <v>15223.4928419187</v>
+        <v>13505.815113867</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6865,23 +6865,23 @@
       </c>
       <c r="E35" s="40" t="n">
         <f aca="false">E28+E34</f>
-        <v>37096.788291617</v>
+        <v>35211.9522249009</v>
       </c>
       <c r="F35" s="40" t="n">
         <f aca="false">F28+F34</f>
-        <v>37410.4914684366</v>
+        <v>35257.884463443</v>
       </c>
       <c r="G35" s="40" t="n">
         <f aca="false">G28+G34</f>
-        <v>37864.6433890555</v>
+        <v>35546.2434262762</v>
       </c>
       <c r="H35" s="40" t="n">
         <f aca="false">H28+H34</f>
-        <v>38292.431026575</v>
+        <v>35521.3975000692</v>
       </c>
       <c r="I35" s="40" t="n">
         <f aca="false">I28+I34</f>
-        <v>38492.9603646005</v>
+        <v>35530.0659041208</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7014,23 +7014,23 @@
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">'Income Statement'!E15</f>
-        <v>3323.7208953</v>
+        <v>1614.342555</v>
       </c>
       <c r="F6" s="10" t="n">
         <f aca="false">'Income Statement'!F15</f>
-        <v>3874.92795691624</v>
+        <v>2405.86606513503</v>
       </c>
       <c r="G6" s="10" t="n">
         <f aca="false">'Income Statement'!G15</f>
-        <v>4465.8093254168</v>
+        <v>3175.05498876406</v>
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">'Income Statement'!H15</f>
-        <v>4998.89045250008</v>
+        <v>3857.44867124394</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">'Income Statement'!I15</f>
-        <v>5275.91483393109</v>
+        <v>4437.15300970018</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7048,23 +7048,23 @@
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">'Income Statement'!E5*Assumptions!E45</f>
-        <v>754.95984</v>
+        <v>679.064</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">'Income Statement'!F5*Assumptions!F45</f>
-        <v>781.7485056</v>
+        <v>691.7930336</v>
       </c>
       <c r="G7" s="10" t="n">
         <f aca="false">'Income Statement'!G5*Assumptions!G45</f>
-        <v>816.412387008</v>
+        <v>722.243943872</v>
       </c>
       <c r="H7" s="10" t="n">
         <f aca="false">'Income Statement'!H5*Assumptions!H45</f>
-        <v>849.81430697472</v>
+        <v>755.14944145728</v>
       </c>
       <c r="I7" s="10" t="n">
         <f aca="false">'Income Statement'!I5*Assumptions!I45</f>
-        <v>882.315494375194</v>
+        <v>786.079595250211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7082,23 +7082,23 @@
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">'Income Statement'!E5*Assumptions!E46</f>
-        <v>707.77485</v>
+        <v>636.6225</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">'Income Statement'!F5*Assumptions!F46</f>
-        <v>732.889224</v>
+        <v>648.555969</v>
       </c>
       <c r="G8" s="10" t="n">
         <f aca="false">'Income Statement'!G5*Assumptions!G46</f>
-        <v>765.38661282</v>
+        <v>677.10369738</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">'Income Statement'!H5*Assumptions!H46</f>
-        <v>796.7009127888</v>
+        <v>707.9526013662</v>
       </c>
       <c r="I8" s="10" t="n">
         <f aca="false">'Income Statement'!I5*Assumptions!I46</f>
-        <v>827.170775976744</v>
+        <v>736.949620547073</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7110,23 +7110,23 @@
       <c r="D9" s="22"/>
       <c r="E9" s="10" t="n">
         <f aca="false">'Balance Sheet'!D8-'Balance Sheet'!E8</f>
-        <v>242.946410958903</v>
+        <v>814.764383561644</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">'Balance Sheet'!E8-'Balance Sheet'!F8</f>
-        <v>65.88967890411</v>
+        <v>141.011744657534</v>
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">'Balance Sheet'!F8-'Balance Sheet'!G8</f>
-        <v>30.2982456986301</v>
+        <v>28.3475438904106</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">'Balance Sheet'!G8-'Balance Sheet'!H8</f>
-        <v>-228.780273744657</v>
+        <v>-225.380120447123</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">'Balance Sheet'!H8-'Balance Sheet'!I8</f>
-        <v>-222.610872605984</v>
+        <v>-211.850368444734</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7138,23 +7138,23 @@
       <c r="D10" s="22"/>
       <c r="E10" s="10" t="n">
         <f aca="false">'Balance Sheet'!D9-'Balance Sheet'!E9</f>
-        <v>132.38512328767</v>
+        <v>815.010273972603</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">'Balance Sheet'!E9-'Balance Sheet'!F9</f>
-        <v>-43.2712114849292</v>
+        <v>68.9419765589037</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">'Balance Sheet'!F9-'Balance Sheet'!G9</f>
-        <v>-103.581364807893</v>
+        <v>-90.9165511509036</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">'Balance Sheet'!G9-'Balance Sheet'!H9</f>
-        <v>-156.871474262332</v>
+        <v>-171.136775669524</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">'Balance Sheet'!H9-'Balance Sheet'!I9</f>
-        <v>-293.428956453763</v>
+        <v>-217.824721582206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7166,23 +7166,23 @@
       <c r="D11" s="22"/>
       <c r="E11" s="10" t="n">
         <f aca="false">'Balance Sheet'!D10-'Balance Sheet'!E10</f>
-        <v>-26.50954</v>
+        <v>191.691</v>
       </c>
       <c r="F11" s="10" t="n">
         <f aca="false">'Balance Sheet'!E10-'Balance Sheet'!F10</f>
-        <v>-77.0174136000001</v>
+        <v>-36.5959716000002</v>
       </c>
       <c r="G11" s="10" t="n">
         <f aca="false">'Balance Sheet'!F10-'Balance Sheet'!G10</f>
-        <v>-99.6586590480001</v>
+        <v>-87.5463670320003</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">'Balance Sheet'!G10-'Balance Sheet'!H10</f>
-        <v>-96.03051990432</v>
+        <v>-94.60330555768</v>
       </c>
       <c r="I11" s="10" t="n">
         <f aca="false">'Balance Sheet'!H10-'Balance Sheet'!I10</f>
-        <v>-93.4409137763619</v>
+        <v>-88.9241921546773</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7194,23 +7194,23 @@
       <c r="D12" s="22"/>
       <c r="E12" s="10" t="n">
         <f aca="false">'Balance Sheet'!E20-'Balance Sheet'!D20</f>
-        <v>84.3074383561652</v>
+        <v>-257.005136986301</v>
       </c>
       <c r="F12" s="10" t="n">
         <f aca="false">'Balance Sheet'!F20-'Balance Sheet'!E20</f>
-        <v>97.2670964383551</v>
+        <v>33.0499071232885</v>
       </c>
       <c r="G12" s="10" t="n">
         <f aca="false">'Balance Sheet'!G20-'Balance Sheet'!F20</f>
-        <v>132.73143031233</v>
+        <v>117.686636435616</v>
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">'Balance Sheet'!H20-'Balance Sheet'!G20</f>
-        <v>123.767154507616</v>
+        <v>126.848107263672</v>
       </c>
       <c r="I12" s="10" t="n">
         <f aca="false">'Balance Sheet'!I20-'Balance Sheet'!H20</f>
-        <v>154.4362928704</v>
+        <v>114.644590306425</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7222,23 +7222,23 @@
       <c r="D13" s="22"/>
       <c r="E13" s="10" t="n">
         <f aca="false">'Balance Sheet'!E21-'Balance Sheet'!D21</f>
-        <v>89.2336900000009</v>
+        <v>-532.1635</v>
       </c>
       <c r="F13" s="10" t="n">
         <f aca="false">'Balance Sheet'!F21-'Balance Sheet'!E21</f>
-        <v>219.3321996</v>
+        <v>104.218962600001</v>
       </c>
       <c r="G13" s="10" t="n">
         <f aca="false">'Balance Sheet'!G21-'Balance Sheet'!F21</f>
-        <v>283.810529028</v>
+        <v>249.316827852</v>
       </c>
       <c r="H13" s="10" t="n">
         <f aca="false">'Balance Sheet'!H21-'Balance Sheet'!G21</f>
-        <v>273.478219727521</v>
+        <v>269.41376147948</v>
       </c>
       <c r="I13" s="10" t="n">
         <f aca="false">'Balance Sheet'!I21-'Balance Sheet'!H21</f>
-        <v>266.103471841378</v>
+        <v>253.240634179624</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7291,23 +7291,23 @@
       </c>
       <c r="E15" s="36" t="n">
         <f aca="false">SUM(E6:E14)</f>
-        <v>5308.81870790274</v>
+        <v>3962.32607554795</v>
       </c>
       <c r="F15" s="36" t="n">
         <f aca="false">SUM(F6:F14)</f>
-        <v>5651.76603637377</v>
+        <v>4056.84168707476</v>
       </c>
       <c r="G15" s="36" t="n">
         <f aca="false">SUM(G6:G14)</f>
-        <v>6291.20850642786</v>
+        <v>4791.29072001118</v>
       </c>
       <c r="H15" s="36" t="n">
         <f aca="false">SUM(H6:H14)</f>
-        <v>6560.96877858743</v>
+        <v>5225.69238113624</v>
       </c>
       <c r="I15" s="36" t="n">
         <f aca="false">SUM(I6:I14)</f>
-        <v>6796.4601261587</v>
+        <v>5809.4681678019</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7338,23 +7338,23 @@
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">-'Income Statement'!E5*Assumptions!E47</f>
-        <v>-754.95984</v>
+        <v>-679.064</v>
       </c>
       <c r="F18" s="10" t="n">
         <f aca="false">-'Income Statement'!F5*Assumptions!F47</f>
-        <v>-781.7485056</v>
+        <v>-691.7930336</v>
       </c>
       <c r="G18" s="10" t="n">
         <f aca="false">-'Income Statement'!G5*Assumptions!G47</f>
-        <v>-816.412387008</v>
+        <v>-722.243943872</v>
       </c>
       <c r="H18" s="10" t="n">
         <f aca="false">-'Income Statement'!H5*Assumptions!H47</f>
-        <v>-849.81430697472</v>
+        <v>-755.14944145728</v>
       </c>
       <c r="I18" s="10" t="n">
         <f aca="false">-'Income Statement'!I5*Assumptions!I47</f>
-        <v>-882.315494375194</v>
+        <v>-786.079595250211</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7407,23 +7407,23 @@
       </c>
       <c r="E20" s="36" t="n">
         <f aca="false">E18+E19</f>
-        <v>-754.95984</v>
+        <v>-679.064</v>
       </c>
       <c r="F20" s="36" t="n">
         <f aca="false">F18+F19</f>
-        <v>-781.7485056</v>
+        <v>-691.7930336</v>
       </c>
       <c r="G20" s="36" t="n">
         <f aca="false">G18+G19</f>
-        <v>-816.412387008</v>
+        <v>-722.243943872</v>
       </c>
       <c r="H20" s="36" t="n">
         <f aca="false">H18+H19</f>
-        <v>-849.81430697472</v>
+        <v>-755.14944145728</v>
       </c>
       <c r="I20" s="36" t="n">
         <f aca="false">I18+I19</f>
-        <v>-882.315494375194</v>
+        <v>-786.079595250211</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7488,23 +7488,23 @@
       </c>
       <c r="E24" s="10" t="n">
         <f aca="false">-'Income Statement'!E19*'Income Statement'!E17</f>
-        <v>-2518.24858203916</v>
+        <v>-2409.84419311276</v>
       </c>
       <c r="F24" s="10" t="n">
         <f aca="false">-'Income Statement'!F19*'Income Statement'!F17</f>
-        <v>-2610.71330013504</v>
+        <v>-2395.75866531623</v>
       </c>
       <c r="G24" s="10" t="n">
         <f aca="false">-'Income Statement'!G19*'Income Statement'!G17</f>
-        <v>-2693.58597695814</v>
+        <v>-2430.80318759847</v>
       </c>
       <c r="H24" s="10" t="n">
         <f aca="false">-'Income Statement'!H19*'Income Statement'!H17</f>
-        <v>-2765.04910200456</v>
+        <v>-2486.50906756031</v>
       </c>
       <c r="I24" s="10" t="n">
         <f aca="false">-'Income Statement'!I19*'Income Statement'!I17</f>
-        <v>-2823.09603659415</v>
+        <v>-2533.31945068174</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7522,23 +7522,23 @@
       </c>
       <c r="E25" s="10" t="n">
         <f aca="false">-Assumptions!E64</f>
-        <v>-1000</v>
+        <v>-250</v>
       </c>
       <c r="F25" s="10" t="n">
         <f aca="false">-Assumptions!F64</f>
-        <v>-2000</v>
+        <v>-750</v>
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">-Assumptions!G64</f>
-        <v>-2500</v>
+        <v>-1500</v>
       </c>
       <c r="H25" s="10" t="n">
         <f aca="false">-Assumptions!H64</f>
-        <v>-3000</v>
+        <v>-2500</v>
       </c>
       <c r="I25" s="10" t="n">
         <f aca="false">-Assumptions!I64</f>
-        <v>-3500</v>
+        <v>-3000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7591,23 +7591,23 @@
       </c>
       <c r="E27" s="36" t="n">
         <f aca="false">SUM(E23:E26)</f>
-        <v>-5518.24858203916</v>
+        <v>-4659.84419311276</v>
       </c>
       <c r="F27" s="36" t="n">
         <f aca="false">SUM(F23:F26)</f>
-        <v>-4610.71330013504</v>
+        <v>-3145.75866531623</v>
       </c>
       <c r="G27" s="36" t="n">
         <f aca="false">SUM(G23:G26)</f>
-        <v>-5193.58597695814</v>
+        <v>-3930.80318759847</v>
       </c>
       <c r="H27" s="36" t="n">
         <f aca="false">SUM(H23:H26)</f>
-        <v>-5765.04910200456</v>
+        <v>-4986.50906756031</v>
       </c>
       <c r="I27" s="36" t="n">
         <f aca="false">SUM(I23:I26)</f>
-        <v>-6323.09603659415</v>
+        <v>-5533.31945068174</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7657,23 +7657,23 @@
       </c>
       <c r="E30" s="36" t="n">
         <f aca="false">E15+E20+E27+E29</f>
-        <v>-964.389714136426</v>
+        <v>-1376.58211756482</v>
       </c>
       <c r="F30" s="36" t="n">
         <f aca="false">F15+F20+F27+F29</f>
-        <v>259.304230638728</v>
+        <v>219.289988158534</v>
       </c>
       <c r="G30" s="36" t="n">
         <f aca="false">G15+G20+G27+G29</f>
-        <v>281.210142461728</v>
+        <v>138.243588540708</v>
       </c>
       <c r="H30" s="36" t="n">
         <f aca="false">H15+H20+H27+H29</f>
-        <v>-53.8946303918456</v>
+        <v>-515.966127881346</v>
       </c>
       <c r="I30" s="36" t="n">
         <f aca="false">I15+I20+I27+I29</f>
-        <v>-408.951404810645</v>
+        <v>-509.930878130057</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7695,19 +7695,19 @@
       </c>
       <c r="F31" s="33" t="n">
         <f aca="false">E32</f>
-        <v>6598.61028586357</v>
+        <v>6186.41788243518</v>
       </c>
       <c r="G31" s="33" t="n">
         <f aca="false">F32</f>
-        <v>6857.9145165023</v>
+        <v>6405.70787059372</v>
       </c>
       <c r="H31" s="33" t="n">
         <f aca="false">G32</f>
-        <v>7139.12465896403</v>
+        <v>6543.95145913443</v>
       </c>
       <c r="I31" s="33" t="n">
         <f aca="false">H32</f>
-        <v>7085.23002857218</v>
+        <v>6027.98533125308</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7728,23 +7728,23 @@
       </c>
       <c r="E32" s="40" t="n">
         <f aca="false">E31+E30</f>
-        <v>6598.61028586357</v>
+        <v>6186.41788243518</v>
       </c>
       <c r="F32" s="40" t="n">
         <f aca="false">F31+F30</f>
-        <v>6857.9145165023</v>
+        <v>6405.70787059372</v>
       </c>
       <c r="G32" s="40" t="n">
         <f aca="false">G31+G30</f>
-        <v>7139.12465896403</v>
+        <v>6543.95145913443</v>
       </c>
       <c r="H32" s="40" t="n">
         <f aca="false">H31+H30</f>
-        <v>7085.23002857218</v>
+        <v>6027.98533125308</v>
       </c>
       <c r="I32" s="40" t="n">
         <f aca="false">I31+I30</f>
-        <v>6676.27862376154</v>
+        <v>5518.05445312302</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7778,23 +7778,23 @@
       </c>
       <c r="E35" s="49" t="n">
         <f aca="false">E15+E18</f>
-        <v>4553.85886790274</v>
+        <v>3283.26207554795</v>
       </c>
       <c r="F35" s="49" t="n">
         <f aca="false">F15+F18</f>
-        <v>4870.01753077377</v>
+        <v>3365.04865347476</v>
       </c>
       <c r="G35" s="49" t="n">
         <f aca="false">G15+G18</f>
-        <v>5474.79611941986</v>
+        <v>4069.04677613918</v>
       </c>
       <c r="H35" s="49" t="n">
         <f aca="false">H15+H18</f>
-        <v>5711.15447161271</v>
+        <v>4470.54293967896</v>
       </c>
       <c r="I35" s="49" t="n">
         <f aca="false">I15+I18</f>
-        <v>5914.14463178351</v>
+        <v>5023.38857255169</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7815,23 +7815,23 @@
       </c>
       <c r="E36" s="33" t="n">
         <f aca="false">-E24-E25</f>
-        <v>3518.24858203916</v>
+        <v>2659.84419311276</v>
       </c>
       <c r="F36" s="33" t="n">
         <f aca="false">-F24-F25</f>
-        <v>4610.71330013504</v>
+        <v>3145.75866531623</v>
       </c>
       <c r="G36" s="33" t="n">
         <f aca="false">-G24-G25</f>
-        <v>5193.58597695814</v>
+        <v>3930.80318759847</v>
       </c>
       <c r="H36" s="33" t="n">
         <f aca="false">-H24-H25</f>
-        <v>5765.04910200456</v>
+        <v>4986.50906756031</v>
       </c>
       <c r="I36" s="33" t="n">
         <f aca="false">-I24-I25</f>
-        <v>6323.09603659415</v>
+        <v>5533.31945068174</v>
       </c>
     </row>
   </sheetData>
@@ -7924,23 +7924,23 @@
       </c>
       <c r="E6" s="33" t="n">
         <f aca="false">D6*(1+Assumptions!E16)</f>
-        <v>21331.44</v>
+        <v>19280.34</v>
       </c>
       <c r="F6" s="33" t="n">
         <f aca="false">E6*(1+Assumptions!F16)</f>
-        <v>22398.012</v>
+        <v>19858.7502</v>
       </c>
       <c r="G6" s="33" t="n">
         <f aca="false">F6*(1+Assumptions!G16)</f>
-        <v>23517.9126</v>
+        <v>20851.68771</v>
       </c>
       <c r="H6" s="33" t="n">
         <f aca="false">G6*(1+Assumptions!H16)</f>
-        <v>24458.629104</v>
+        <v>21894.2720955</v>
       </c>
       <c r="I6" s="33" t="n">
         <f aca="false">H6*(1+Assumptions!I16)</f>
-        <v>25436.97426816</v>
+        <v>22770.04297932</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7958,23 +7958,23 @@
       </c>
       <c r="E7" s="33" t="n">
         <f aca="false">D7*(1+Assumptions!E17)</f>
-        <v>12823.44</v>
+        <v>11566.24</v>
       </c>
       <c r="F7" s="33" t="n">
         <f aca="false">E7*(1+Assumptions!F17)</f>
-        <v>13208.1432</v>
+        <v>11797.5648</v>
       </c>
       <c r="G7" s="33" t="n">
         <f aca="false">F7*(1+Assumptions!G17)</f>
-        <v>13736.468928</v>
+        <v>12269.467392</v>
       </c>
       <c r="H7" s="33" t="n">
         <f aca="false">G7*(1+Assumptions!H17)</f>
-        <v>14285.92768512</v>
+        <v>12760.24608768</v>
       </c>
       <c r="I7" s="33" t="n">
         <f aca="false">H7*(1+Assumptions!I17)</f>
-        <v>14714.5055156736</v>
+        <v>13270.6559311872</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7992,23 +7992,23 @@
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">D8*(1+Assumptions!E18)</f>
-        <v>5554.65</v>
+        <v>4677.6</v>
       </c>
       <c r="F8" s="33" t="n">
         <f aca="false">E8*(1+Assumptions!F18)</f>
-        <v>5554.65</v>
+        <v>4537.272</v>
       </c>
       <c r="G8" s="33" t="n">
         <f aca="false">F8*(1+Assumptions!G18)</f>
-        <v>5721.2895</v>
+        <v>4673.39016</v>
       </c>
       <c r="H8" s="33" t="n">
         <f aca="false">G8*(1+Assumptions!H18)</f>
-        <v>5950.14108</v>
+        <v>4860.3257664</v>
       </c>
       <c r="I8" s="33" t="n">
         <f aca="false">H8*(1+Assumptions!I18)</f>
-        <v>6188.1467232</v>
+        <v>5054.738797056</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8026,23 +8026,23 @@
       </c>
       <c r="E9" s="33" t="n">
         <f aca="false">D9*(1+Assumptions!E19)</f>
-        <v>6367.86</v>
+        <v>5868.42</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">E9*(1+Assumptions!F19)</f>
-        <v>6622.5744</v>
+        <v>6044.4726</v>
       </c>
       <c r="G9" s="33" t="n">
         <f aca="false">F9*(1+Assumptions!G19)</f>
-        <v>6953.70312</v>
+        <v>6346.69623</v>
       </c>
       <c r="H9" s="33" t="n">
         <f aca="false">G9*(1+Assumptions!H19)</f>
-        <v>7301.388276</v>
+        <v>6664.0310415</v>
       </c>
       <c r="I9" s="33" t="n">
         <f aca="false">H9*(1+Assumptions!I19)</f>
-        <v>7666.4576898</v>
+        <v>6997.232593575</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8060,23 +8060,23 @@
       </c>
       <c r="E10" s="33" t="n">
         <f aca="false">D10*(1+Assumptions!E20)</f>
-        <v>1056.6</v>
+        <v>997.9</v>
       </c>
       <c r="F10" s="33" t="n">
         <f aca="false">E10*(1+Assumptions!F20)</f>
-        <v>1024.902</v>
+        <v>948.005</v>
       </c>
       <c r="G10" s="33" t="n">
         <f aca="false">F10*(1+Assumptions!G20)</f>
-        <v>1045.40004</v>
+        <v>948.005</v>
       </c>
       <c r="H10" s="33" t="n">
         <f aca="false">G10*(1+Assumptions!H20)</f>
-        <v>1066.3080408</v>
+        <v>966.9651</v>
       </c>
       <c r="I10" s="33" t="n">
         <f aca="false">H10*(1+Assumptions!I20)</f>
-        <v>1087.634201616</v>
+        <v>986.304402</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8091,23 +8091,23 @@
       </c>
       <c r="E11" s="36" t="n">
         <f aca="false">SUM(E6:E10)+Assumptions!E36</f>
-        <v>47184.99</v>
+        <v>42441.5</v>
       </c>
       <c r="F11" s="36" t="n">
         <f aca="false">SUM(F6:F10)+Assumptions!F36</f>
-        <v>48859.2816</v>
+        <v>43237.0646</v>
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">SUM(G6:G10)+Assumptions!G36</f>
-        <v>51025.774188</v>
+        <v>45140.246492</v>
       </c>
       <c r="H11" s="36" t="n">
         <f aca="false">SUM(H6:H10)+Assumptions!H36</f>
-        <v>53113.39418592</v>
+        <v>47196.84009108</v>
       </c>
       <c r="I11" s="36" t="n">
         <f aca="false">SUM(I6:I10)+Assumptions!I36</f>
-        <v>55144.7183984496</v>
+        <v>49129.9747031382</v>
       </c>
       <c r="K11" s="51" t="s">
         <v>178</v>
@@ -8125,23 +8125,23 @@
       </c>
       <c r="E12" s="49" t="n">
         <f aca="false">E11*(Assumptions!E39-Assumptions!E43-Assumptions!E44)</f>
-        <v>4105.09413</v>
+        <v>1994.7505</v>
       </c>
       <c r="F12" s="49" t="n">
         <f aca="false">F11*(Assumptions!F39-Assumptions!F43-Assumptions!F44)</f>
-        <v>4739.3503152</v>
+        <v>2940.1203928</v>
       </c>
       <c r="G12" s="49" t="n">
         <f aca="false">G11*(Assumptions!G39-Assumptions!G43-Assumptions!G44)</f>
-        <v>5459.757838116</v>
+        <v>3882.061198312</v>
       </c>
       <c r="H12" s="49" t="n">
         <f aca="false">H11*(Assumptions!H39-Assumptions!H43-Assumptions!H44)</f>
-        <v>6108.0403313808</v>
+        <v>4719.684009108</v>
       </c>
       <c r="I12" s="49" t="n">
         <f aca="false">I11*(Assumptions!I39-Assumptions!I43-Assumptions!I44)</f>
-        <v>6451.9320526186</v>
+        <v>5453.42719204834</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8156,23 +8156,23 @@
       </c>
       <c r="E13" s="37" t="n">
         <f aca="false">E12/E11</f>
-        <v>0.087</v>
+        <v>0.047</v>
       </c>
       <c r="F13" s="37" t="n">
         <f aca="false">F12/F11</f>
-        <v>0.097</v>
+        <v>0.068</v>
       </c>
       <c r="G13" s="37" t="n">
         <f aca="false">G12/G11</f>
-        <v>0.107</v>
+        <v>0.086</v>
       </c>
       <c r="H13" s="37" t="n">
         <f aca="false">H12/H11</f>
-        <v>0.115</v>
+        <v>0.1</v>
       </c>
       <c r="I13" s="37" t="n">
         <f aca="false">I12/I11</f>
-        <v>0.117</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8203,23 +8203,23 @@
       </c>
       <c r="E16" s="33" t="n">
         <f aca="false">D16*(1+Assumptions!E23)</f>
-        <v>21741.66</v>
+        <v>19895.67</v>
       </c>
       <c r="F16" s="33" t="n">
         <f aca="false">E16*(1+Assumptions!F23)</f>
-        <v>23263.5762</v>
+        <v>20890.4535</v>
       </c>
       <c r="G16" s="33" t="n">
         <f aca="false">F16*(1+Assumptions!G23)</f>
-        <v>24892.026534</v>
+        <v>22352.785245</v>
       </c>
       <c r="H16" s="33" t="n">
         <f aca="false">G16*(1+Assumptions!H23)</f>
-        <v>26385.54812604</v>
+        <v>23693.9523597</v>
       </c>
       <c r="I16" s="33" t="n">
         <f aca="false">H16*(1+Assumptions!I23)</f>
-        <v>27704.825532342</v>
+        <v>24878.649977685</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8237,23 +8237,23 @@
       </c>
       <c r="E17" s="33" t="n">
         <f aca="false">D17*(1+Assumptions!E24)</f>
-        <v>13074.88</v>
+        <v>11943.4</v>
       </c>
       <c r="F17" s="33" t="n">
         <f aca="false">E17*(1+Assumptions!F24)</f>
-        <v>13728.624</v>
+        <v>12421.136</v>
       </c>
       <c r="G17" s="33" t="n">
         <f aca="false">F17*(1+Assumptions!G24)</f>
-        <v>14552.34144</v>
+        <v>13166.40416</v>
       </c>
       <c r="H17" s="33" t="n">
         <f aca="false">G17*(1+Assumptions!H24)</f>
-        <v>15279.958512</v>
+        <v>13824.724368</v>
       </c>
       <c r="I17" s="33" t="n">
         <f aca="false">H17*(1+Assumptions!I24)</f>
-        <v>15891.15685248</v>
+        <v>14515.9605864</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8271,23 +8271,23 @@
       </c>
       <c r="E18" s="33" t="n">
         <f aca="false">D18*(1+Assumptions!E25)</f>
-        <v>5847</v>
+        <v>4969.95</v>
       </c>
       <c r="F18" s="33" t="n">
         <f aca="false">E18*(1+Assumptions!F25)</f>
-        <v>6139.35</v>
+        <v>5119.0485</v>
       </c>
       <c r="G18" s="33" t="n">
         <f aca="false">F18*(1+Assumptions!G25)</f>
-        <v>6507.711</v>
+        <v>5426.19141</v>
       </c>
       <c r="H18" s="33" t="n">
         <f aca="false">G18*(1+Assumptions!H25)</f>
-        <v>6898.17366</v>
+        <v>5751.7628946</v>
       </c>
       <c r="I18" s="33" t="n">
         <f aca="false">H18*(1+Assumptions!I25)</f>
-        <v>7243.082343</v>
+        <v>6039.35103933</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8305,23 +8305,23 @@
       </c>
       <c r="E19" s="33" t="n">
         <f aca="false">D19*(1+Assumptions!E26)</f>
-        <v>6492.72</v>
+        <v>6055.71</v>
       </c>
       <c r="F19" s="33" t="n">
         <f aca="false">E19*(1+Assumptions!F26)</f>
-        <v>6882.2832</v>
+        <v>6358.4955</v>
       </c>
       <c r="G19" s="33" t="n">
         <f aca="false">F19*(1+Assumptions!G26)</f>
-        <v>7364.043024</v>
+        <v>6803.590185</v>
       </c>
       <c r="H19" s="33" t="n">
         <f aca="false">G19*(1+Assumptions!H26)</f>
-        <v>7879.52603568</v>
+        <v>7279.84149795</v>
       </c>
       <c r="I19" s="33" t="n">
         <f aca="false">H19*(1+Assumptions!I26)</f>
-        <v>8352.2975978208</v>
+        <v>7716.631987827</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8339,23 +8339,23 @@
       </c>
       <c r="E20" s="33" t="n">
         <f aca="false">D20*(1+Assumptions!E27)</f>
-        <v>1115.3</v>
+        <v>1056.6</v>
       </c>
       <c r="F20" s="33" t="n">
         <f aca="false">E20*(1+Assumptions!F27)</f>
-        <v>1137.606</v>
+        <v>1056.6</v>
       </c>
       <c r="G20" s="33" t="n">
         <f aca="false">F20*(1+Assumptions!G27)</f>
-        <v>1183.11024</v>
+        <v>1088.298</v>
       </c>
       <c r="H20" s="33" t="n">
         <f aca="false">G20*(1+Assumptions!H27)</f>
-        <v>1230.4346496</v>
+        <v>1131.82992</v>
       </c>
       <c r="I20" s="33" t="n">
         <f aca="false">H20*(1+Assumptions!I27)</f>
-        <v>1267.347689088</v>
+        <v>1165.7848176</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8370,23 +8370,23 @@
       </c>
       <c r="E21" s="36" t="n">
         <f aca="false">SUM(E16:E20)+Assumptions!E36</f>
-        <v>48322.56</v>
+        <v>43972.33</v>
       </c>
       <c r="F21" s="36" t="n">
         <f aca="false">SUM(F16:F20)+Assumptions!F36</f>
-        <v>51202.4394</v>
+        <v>45896.7335</v>
       </c>
       <c r="G21" s="36" t="n">
         <f aca="false">SUM(G16:G20)+Assumptions!G36</f>
-        <v>54550.232238</v>
+        <v>48888.269</v>
       </c>
       <c r="H21" s="36" t="n">
         <f aca="false">SUM(H16:H20)+Assumptions!H36</f>
-        <v>57724.64098332</v>
+        <v>51733.11104025</v>
       </c>
       <c r="I21" s="36" t="n">
         <f aca="false">SUM(I16:I20)+Assumptions!I36</f>
-        <v>60509.7100147308</v>
+        <v>54367.378408842</v>
       </c>
       <c r="K21" s="51" t="s">
         <v>179</v>
@@ -8404,23 +8404,23 @@
       </c>
       <c r="E22" s="49" t="n">
         <f aca="false">E21*(Assumptions!E40-Assumptions!E43-Assumptions!E44)</f>
-        <v>4445.67552</v>
+        <v>2286.56116</v>
       </c>
       <c r="F22" s="49" t="n">
         <f aca="false">F21*(Assumptions!F40-Assumptions!F43-Assumptions!F44)</f>
-        <v>5478.6610158</v>
+        <v>3579.945213</v>
       </c>
       <c r="G22" s="49" t="n">
         <f aca="false">G21*(Assumptions!G40-Assumptions!G43-Assumptions!G44)</f>
-        <v>6655.128333036</v>
+        <v>4937.715169</v>
       </c>
       <c r="H22" s="49" t="n">
         <f aca="false">H21*(Assumptions!H40-Assumptions!H43-Assumptions!H44)</f>
-        <v>7504.2033278316</v>
+        <v>5949.30776962875</v>
       </c>
       <c r="I22" s="49" t="n">
         <f aca="false">I21*(Assumptions!I40-Assumptions!I43-Assumptions!I44)</f>
-        <v>7987.28172194447</v>
+        <v>6850.28967951409</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8435,23 +8435,23 @@
       </c>
       <c r="E23" s="37" t="n">
         <f aca="false">E22/E21</f>
-        <v>0.092</v>
+        <v>0.052</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">F22/F21</f>
-        <v>0.107</v>
+        <v>0.078</v>
       </c>
       <c r="G23" s="37" t="n">
         <f aca="false">G22/G21</f>
-        <v>0.122</v>
+        <v>0.101</v>
       </c>
       <c r="H23" s="37" t="n">
         <f aca="false">H22/H21</f>
-        <v>0.13</v>
+        <v>0.115</v>
       </c>
       <c r="I23" s="37" t="n">
         <f aca="false">I22/I21</f>
-        <v>0.132</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8482,23 +8482,23 @@
       </c>
       <c r="E26" s="33" t="n">
         <f aca="false">D26*(1+Assumptions!E30)</f>
-        <v>20716.11</v>
+        <v>18665.01</v>
       </c>
       <c r="F26" s="33" t="n">
         <f aca="false">E26*(1+Assumptions!F30)</f>
-        <v>21130.4322</v>
+        <v>18665.01</v>
       </c>
       <c r="G26" s="33" t="n">
         <f aca="false">F26*(1+Assumptions!G30)</f>
-        <v>21553.040844</v>
+        <v>19038.3102</v>
       </c>
       <c r="H26" s="33" t="n">
         <f aca="false">G26*(1+Assumptions!H30)</f>
-        <v>21984.10166088</v>
+        <v>19609.459506</v>
       </c>
       <c r="I26" s="33" t="n">
         <f aca="false">H26*(1+Assumptions!I30)</f>
-        <v>22423.7836940976</v>
+        <v>20197.74329118</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8516,23 +8516,23 @@
       </c>
       <c r="E27" s="33" t="n">
         <f aca="false">D27*(1+Assumptions!E31)</f>
-        <v>12320.56</v>
+        <v>11189.08</v>
       </c>
       <c r="F27" s="33" t="n">
         <f aca="false">E27*(1+Assumptions!F31)</f>
-        <v>12320.56</v>
+        <v>10965.2984</v>
       </c>
       <c r="G27" s="33" t="n">
         <f aca="false">F27*(1+Assumptions!G31)</f>
-        <v>12443.7656</v>
+        <v>11074.951384</v>
       </c>
       <c r="H27" s="33" t="n">
         <f aca="false">G27*(1+Assumptions!H31)</f>
-        <v>12692.640912</v>
+        <v>11296.45041168</v>
       </c>
       <c r="I27" s="33" t="n">
         <f aca="false">H27*(1+Assumptions!I31)</f>
-        <v>12946.49373024</v>
+        <v>11522.3794199136</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8550,23 +8550,23 @@
       </c>
       <c r="E28" s="33" t="n">
         <f aca="false">D28*(1+Assumptions!E32)</f>
-        <v>5145.36</v>
+        <v>4326.78</v>
       </c>
       <c r="F28" s="33" t="n">
         <f aca="false">E28*(1+Assumptions!F32)</f>
-        <v>4836.6384</v>
+        <v>3894.102</v>
       </c>
       <c r="G28" s="33" t="n">
         <f aca="false">F28*(1+Assumptions!G32)</f>
-        <v>4739.905632</v>
+        <v>3777.27894</v>
       </c>
       <c r="H28" s="33" t="n">
         <f aca="false">G28*(1+Assumptions!H32)</f>
-        <v>4739.905632</v>
+        <v>3777.27894</v>
       </c>
       <c r="I28" s="33" t="n">
         <f aca="false">H28*(1+Assumptions!I32)</f>
-        <v>4787.30468832</v>
+        <v>3815.0517294</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8584,23 +8584,23 @@
       </c>
       <c r="E29" s="33" t="n">
         <f aca="false">D29*(1+Assumptions!E33)</f>
-        <v>6180.57</v>
+        <v>5681.13</v>
       </c>
       <c r="F29" s="33" t="n">
         <f aca="false">E29*(1+Assumptions!F33)</f>
-        <v>6242.3757</v>
+        <v>5681.13</v>
       </c>
       <c r="G29" s="33" t="n">
         <f aca="false">F29*(1+Assumptions!G33)</f>
-        <v>6367.223214</v>
+        <v>5794.7526</v>
       </c>
       <c r="H29" s="33" t="n">
         <f aca="false">G29*(1+Assumptions!H33)</f>
-        <v>6558.23991042</v>
+        <v>5968.595178</v>
       </c>
       <c r="I29" s="33" t="n">
         <f aca="false">H29*(1+Assumptions!I33)</f>
-        <v>6754.9871077326</v>
+        <v>6147.65303334</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8618,23 +8618,23 @@
       </c>
       <c r="E30" s="33" t="n">
         <f aca="false">D30*(1+Assumptions!E34)</f>
-        <v>962.68</v>
+        <v>939.2</v>
       </c>
       <c r="F30" s="33" t="n">
         <f aca="false">E30*(1+Assumptions!F34)</f>
-        <v>885.6656</v>
+        <v>845.28</v>
       </c>
       <c r="G30" s="33" t="n">
         <f aca="false">F30*(1+Assumptions!G34)</f>
-        <v>859.095632</v>
+        <v>819.9216</v>
       </c>
       <c r="H30" s="33" t="n">
         <f aca="false">G30*(1+Assumptions!H34)</f>
-        <v>859.095632</v>
+        <v>819.9216</v>
       </c>
       <c r="I30" s="33" t="n">
         <f aca="false">H30*(1+Assumptions!I34)</f>
-        <v>859.095632</v>
+        <v>819.9216</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8649,23 +8649,23 @@
       </c>
       <c r="E31" s="36" t="n">
         <f aca="false">SUM(E26:E30)+Assumptions!E36</f>
-        <v>45376.28</v>
+        <v>40852.2</v>
       </c>
       <c r="F31" s="36" t="n">
         <f aca="false">SUM(F26:F30)+Assumptions!F36</f>
-        <v>45466.6719</v>
+        <v>40101.8204</v>
       </c>
       <c r="G31" s="36" t="n">
         <f aca="false">SUM(G26:G30)+Assumptions!G36</f>
-        <v>46014.030922</v>
+        <v>40556.214724</v>
       </c>
       <c r="H31" s="36" t="n">
         <f aca="false">SUM(H26:H30)+Assumptions!H36</f>
-        <v>46884.9837473</v>
+        <v>41522.70563568</v>
       </c>
       <c r="I31" s="36" t="n">
         <f aca="false">SUM(I26:I30)+Assumptions!I36</f>
-        <v>47822.6648523902</v>
+        <v>42553.7490738336</v>
       </c>
       <c r="K31" s="51" t="s">
         <v>180</v>
@@ -8683,23 +8683,23 @@
       </c>
       <c r="E32" s="49" t="n">
         <f aca="false">E31*(Assumptions!E41-Assumptions!E43-Assumptions!E44)</f>
-        <v>3720.85496</v>
+        <v>1715.7924</v>
       </c>
       <c r="F32" s="49" t="n">
         <f aca="false">F31*(Assumptions!F41-Assumptions!F43-Assumptions!F44)</f>
-        <v>3955.6004553</v>
+        <v>2325.9055832</v>
       </c>
       <c r="G32" s="49" t="n">
         <f aca="false">G31*(Assumptions!G41-Assumptions!G43-Assumptions!G44)</f>
-        <v>4371.33293759</v>
+        <v>3082.272319024</v>
       </c>
       <c r="H32" s="49" t="n">
         <f aca="false">H31*(Assumptions!H41-Assumptions!H43-Assumptions!H44)</f>
-        <v>4688.49837473</v>
+        <v>3737.0435072112</v>
       </c>
       <c r="I32" s="49" t="n">
         <f aca="false">I31*(Assumptions!I41-Assumptions!I43-Assumptions!I44)</f>
-        <v>4877.9118149438</v>
+        <v>4085.15991108803</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8714,23 +8714,23 @@
       </c>
       <c r="E33" s="37" t="n">
         <f aca="false">E32/E31</f>
-        <v>0.082</v>
+        <v>0.042</v>
       </c>
       <c r="F33" s="37" t="n">
         <f aca="false">F32/F31</f>
-        <v>0.087</v>
+        <v>0.058</v>
       </c>
       <c r="G33" s="37" t="n">
         <f aca="false">G32/G31</f>
-        <v>0.095</v>
+        <v>0.076</v>
       </c>
       <c r="H33" s="37" t="n">
         <f aca="false">H32/H31</f>
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="I33" s="37" t="n">
         <f aca="false">I32/I31</f>
-        <v>0.102</v>
+        <v>0.096</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8772,19 +8772,19 @@
       </c>
       <c r="B37" s="54" t="n">
         <f aca="false">I11</f>
-        <v>55144.7183984496</v>
+        <v>49129.9747031382</v>
       </c>
       <c r="C37" s="55" t="n">
         <f aca="false">(I11/D11)^(1/5)-1</f>
-        <v>0.0351443894114794</v>
+        <v>0.0115083121973893</v>
       </c>
       <c r="D37" s="54" t="n">
         <f aca="false">I12</f>
-        <v>6451.9320526186</v>
+        <v>5453.42719204834</v>
       </c>
       <c r="E37" s="55" t="n">
         <f aca="false">I13</f>
-        <v>0.117</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8793,19 +8793,19 @@
       </c>
       <c r="B38" s="54" t="n">
         <f aca="false">I21</f>
-        <v>60509.7100147308</v>
+        <v>54367.378408842</v>
       </c>
       <c r="C38" s="55" t="n">
         <f aca="false">(I21/D21)^(1/5)-1</f>
-        <v>0.054545110098323</v>
+        <v>0.032209439279584</v>
       </c>
       <c r="D38" s="54" t="n">
         <f aca="false">I22</f>
-        <v>7987.28172194447</v>
+        <v>6850.28967951409</v>
       </c>
       <c r="E38" s="55" t="n">
         <f aca="false">I23</f>
-        <v>0.132</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8814,19 +8814,19 @@
       </c>
       <c r="B39" s="54" t="n">
         <f aca="false">I31</f>
-        <v>47822.6648523902</v>
+        <v>42553.7490738336</v>
       </c>
       <c r="C39" s="55" t="n">
         <f aca="false">(I31/D31)^(1/5)-1</f>
-        <v>0.00606699659318721</v>
+        <v>-0.0171489328173601</v>
       </c>
       <c r="D39" s="54" t="n">
         <f aca="false">I32</f>
-        <v>4877.9118149438</v>
+        <v>4085.15991108803</v>
       </c>
       <c r="E39" s="55" t="n">
         <f aca="false">I33</f>
-        <v>0.102</v>
+        <v>0.096</v>
       </c>
     </row>
   </sheetData>

</xml_diff>